<commit_message>
Finanzmodell: Gründerangebot 10 % für 250.000 € (2,25 Mio € Pre-Money), Gründer-Sicht-Bewertung mit vier Methoden, SAFE-Cap 2,25 Mio € ohne Zins
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01STcnjfrFEd99DGQ7JM2gQ3
</commit_message>
<xml_diff>
--- a/live-fx/business/LiveFX_Finanzmodell.xlsx
+++ b/live-fx/business/LiveFX_Finanzmodell.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="590">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1063" uniqueCount="710">
   <si>
     <t xml:space="preserve">LiveFX – Finanzmodell Pre-Seed 250.000 € · Annahmen</t>
   </si>
@@ -1122,124 +1122,148 @@
     <t xml:space="preserve">Lesart: Gate erfüllt, wenn mindestens die Schwelle (konservatives Szenario) erreicht ist; das Ziel ist das Basis-Szenario.</t>
   </si>
   <si>
-    <t xml:space="preserve">Bewertung Pre-Seed – drei Methoden (Vorschlag – mit Steuer-/Rechtsberater prüfen)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alle Eingaben blau; Quellen in Spalte G. Keine Umsätze, Produkt v2.1 funktionsfähig; Solo-Gründer + Investor Relations.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Berkus-Methode (5 Faktoren × max. 500.000 €)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Max. €</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Score (0–1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wert €</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Begründung (ehrlich)</t>
+    <t xml:space="preserve">Bewertung Pre-Seed – Referenzmethoden (Investorensicht) und Angebot der Gründer (Vorschlag – mit Steuer-/Rechtsberater prüfen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alle Eingaben blau; Quellen in Spalte G. „Gründer-Sicht“ = bewusst großzügig gerechnet, jede Annahme belegt und als Gründer-Annahme gekennzeichnet; „konservativ“ = frühere Investorensicht zum Vergleich. Keine Umsätze, Produkt v2.1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teil A (1–5): Referenzmethoden (Investorensicht) – Berkus, Scorecard, VC-Methode, Risk Factor Summation. Teil B (6–10): Angebot der Gründer, Verhandlungsspanne, 10×-Prüfung, Begründung, Wandeldarlehen/SAFE. $→€ jeweils 1:1 (Annahme).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Referenzmethode (Investorensicht): Berkus – Gründer-Sicht und konservativ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max. € je Faktor – Gründer-Sicht (moderne „moderate 2×“-Variante)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gründer-Annahme: moderne Berkus-Anpassung „moderat (2×)“ mit 0–1 Mio. $ je Faktor, max. 5 Mio. $ (valu.vc 2026; icanpitch 2026). Begründung: Berkus zuletzt 2016 aktualisiert, Seed-Bewertungen seitdem deutlich gestiegen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max. € je Faktor – konservativ (klassisch, Dave Berkus)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Original-Methode: bis 0,5 Mio. $ je Faktor, max. 2,5 Mio. $ (berkus.com).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Score Gründer (0–1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wert Gründer €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Score konservativ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wert konservativ €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Begründung (Gründer-Sicht · konservativ)</t>
   </si>
   <si>
     <t xml:space="preserve">Idee / Grundwert (Problem, Markt)</t>
   </si>
   <si>
-    <t xml:space="preserve">Neuer Auslöser Stimme → Effekt; großer Markt (BP §6), aber Zahlungsbereitschaft unbewiesen.</t>
+    <t xml:space="preserve">Hoch: neuer Auslöser Stimme → Effekt, großer Markt (BP §6) · konservativ: Zahlungsbereitschaft unbewiesen.</t>
   </si>
   <si>
     <t xml:space="preserve">Prototyp / Produkt (Technologierisiko)</t>
   </si>
   <si>
-    <t xml:space="preserve">v2.1 funktionsfähig: 238 Trigger + 143 freie Sticker, Leistungsmodus (Bildzeit −63 bis −69 %), sichere GIF-Suche, automatisierte Tests, im Einsatz in eigenen Streams.</t>
+    <t xml:space="preserve">Hoch: v2.1 funktionsfähig und getestet (575+ automatisierte Tests, e2e-Suite), 238 Trigger + 143 freie Sticker, Leistungsmodus, sichere GIF-Suche, im Einsatz in eigenen Streams · nicht 1,0: noch keine zahlenden Nutzer.</t>
   </si>
   <si>
     <t xml:space="preserve">Team (Umsetzungsqualität)</t>
   </si>
   <si>
-    <t xml:space="preserve">Solo-Gründer + Investor Relations; erste Einstellung offen; Ein-Personen-Risiko (BP §13).</t>
+    <t xml:space="preserve">Mittel: Gründer hat Produkt allein bis v2.1 gebaut + Investor Relations · konservativ: Solo-Gründer, Ein-Personen-Risiko (BP §13).</t>
   </si>
   <si>
     <t xml:space="preserve">Strategische Beziehungen</t>
   </si>
   <si>
-    <t xml:space="preserve">Noch keine Plattform-, Bildungs- oder Vertriebspartnerschaft unterzeichnet.</t>
+    <t xml:space="preserve">Niedrig–mittel: eigene TR-Community, Gespräche mit Plattform-/Bildungspartnern geplant · keine Partnerschaft unterzeichnet.</t>
   </si>
   <si>
     <t xml:space="preserve">Produkteinführung / Umsatz</t>
   </si>
   <si>
-    <t xml:space="preserve">Noch kein Umsatz, keine zahlenden Nutzer; Pro-Abo erst ab Monat 3.</t>
+    <t xml:space="preserve">Niedrig (beide Sichten): noch kein Umsatz; Pro-Abo ab Monat 3.</t>
   </si>
   <si>
     <t xml:space="preserve">Berkus-Wert (Pre-Money)</t>
   </si>
   <si>
-    <t xml:space="preserve">Methode: Dave Berkus, je Faktor bis 0,5 Mio. € (Pre-Revenue).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Scorecard-Methode (Payne) – Referenz: Median-Pre-Money Pre-Seed DACH/Türkiye</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Referenz Median-Pre-Money Pre-Seed (pre-revenue, DACH/TR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abgeleitet: DE Pre-Seed typ. 0,5–1,5 Mio. € (upxcale.de), DE 1–5 Mio. € (capvisory.de); Europa Median Q1 2025 4,57 Mio. USD (Equidam, institutionelle Runden, daher zu hoch für Solo-pre-revenue); Türkiye niedriger → 1,5 Mio. € (Schätzung).</t>
+    <t xml:space="preserve">2. Referenzmethode (Investorensicht): Scorecard (Payne) – Gründer-Sicht und konservativ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referenz-Pre-Money Pre-Seed – Gründer-Sicht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gründer-Annahme 2,5 Mio. €: im unteren Teil der DACH-Pre-Seed-Spanne 1,5–5 Mio. € (upxcale; Mitte wäre 3,25 Mio. €) und DE 1–5 Mio. € (capvisory; Mitte 3 Mio. €), deutlich unter dem Europa-Median 4,57 Mio. $ ≈ 4,2 Mio. € (Equidam Q1 2025).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referenz-Pre-Money Pre-Seed – konservativ (DACH/TR, Solo, pre-revenue)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DE Pre-Seed typ. 0,5–1,5 Mio. € (upxcale); Türkiye niedriger → 1,5 Mio. € (Schätzung, frühere Investorensicht).</t>
   </si>
   <si>
     <t xml:space="preserve">Gewicht</t>
   </si>
   <si>
-    <t xml:space="preserve">Vergleich (100 % = Median)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beitrag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Begründung</t>
+    <t xml:space="preserve">Vergleich Gründer (100 % = Referenz)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beitrag Gründer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vergleich konservativ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beitrag konservativ</t>
   </si>
   <si>
     <t xml:space="preserve">Team</t>
   </si>
   <si>
-    <t xml:space="preserve">Solo-Gründer, Hires offen; Produkt- und Community-Erfahrung als Streamer/Autor</t>
+    <t xml:space="preserve">Durchschnitt: Produkt bis v2.1 allein gebaut, Streamer/Autor mit Community · konservativ: Solo, Hires offen</t>
   </si>
   <si>
     <t xml:space="preserve">Marktgröße / Chance</t>
   </si>
   <si>
-    <t xml:space="preserve">Live-Streaming 97–157 Mrd. USD, SAM 1–3 Mio. Creator (BP §6); Vision-Märkte zusätzlich</t>
+    <t xml:space="preserve">Stark: Live-Streaming 97–157 Mrd. USD, SAM 1–3 Mio. Creator (BP §6) + Vision-Märkte A–D</t>
   </si>
   <si>
     <t xml:space="preserve">Produkt / Technologie</t>
   </si>
   <si>
-    <t xml:space="preserve">funktionsfähige v2.1, lokale Verarbeitung, Tests; geringe Grenzkosten</t>
+    <t xml:space="preserve">Stark: ausgeliefertes v2.1 mit 575+ Tests und e2e-Suite, lokale Verarbeitung, geringe Grenzkosten</t>
   </si>
   <si>
     <t xml:space="preserve">Wettbewerbsumfeld</t>
   </si>
   <si>
-    <t xml:space="preserve">kein direkter Sprach-Trigger-Wettbewerber, aber Plattformen können nachbauen</t>
+    <t xml:space="preserve">Günstig: kein direkter Sprach-Trigger-Wettbewerber (Nische) · Risiko: Plattformen können nachbauen</t>
   </si>
   <si>
     <t xml:space="preserve">Marketing / Vertrieb / Partner</t>
   </si>
   <si>
-    <t xml:space="preserve">eigene Streams + TR-Community; noch keine Partner, kein Vertrieb</t>
+    <t xml:space="preserve">Unter Durchschnitt: eigene Streams + TR-Community, noch keine Partner/Vertrieb</t>
   </si>
   <si>
     <t xml:space="preserve">Bedarf weiterer Finanzierung</t>
   </si>
   <si>
-    <t xml:space="preserve">schlanke Runde mit Gates; Folgerunde nötig (siehe Liquidität)</t>
+    <t xml:space="preserve">Neutral: schlanke Runde mit Gates; Folgerunde nötig (siehe Liquidität)</t>
   </si>
   <si>
     <t xml:space="preserve">Sonstiges (IP, Bildung, Datenschutz lokal)</t>
   </si>
   <si>
-    <t xml:space="preserve">WortBild/Bildung als zweites Standbein, offline-fähig</t>
+    <t xml:space="preserve">Eigene Inhalte/IP, WortBild als zweites Standbein, offline-fähig</t>
   </si>
   <si>
     <t xml:space="preserve">Summe Gewichte / Faktor</t>
@@ -1248,37 +1272,46 @@
     <t xml:space="preserve">Scorecard-Wert (Pre-Money)</t>
   </si>
   <si>
-    <t xml:space="preserve">3. VC-Methode (Exit Jahr 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Umsatz J5 (Basis, aus GuV)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GuV 5 Jahre, Basis J5</t>
+    <t xml:space="preserve">3. Referenzmethode (Investorensicht): VC-Methode (Exit Jahr 5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gründer: Optimistisch (Upside)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gründer: Basis (2. Linie)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Konservativ: Basis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quelle / Kennzeichnung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umsatz J5 (aus GuV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GuV 5 Jahre, J5 (2031): optimistisches bzw. Basis-Szenario</t>
   </si>
   <si>
     <t xml:space="preserve">Exit-Multiple (Umsatz)</t>
   </si>
   <si>
-    <t xml:space="preserve">SaaS Capital 2025: private B2B-SaaS 4,8x (bootstrapped) / 5,3x (VC-finanziert); unter 2 Mio. USD ARR 2–3,5x. Abschlag für B2C/Creator-Tool (höherer Churn) → 4,0x (konservativ).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exit-Wert Jahr 5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Umsatz × Multiple</t>
+    <t xml:space="preserve">Gründer-Annahme 6,0x: SaaS Capital 2025 – VC-finanzierte private SaaS 5,3x (bootstrapped 4,8x) + Wachstumsaufschlag; konservativ 4,0x (B2C-/Creator-Abschlag, unter 2 Mio. USD ARR 2–3,5x).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exit-Wert Jahr 5 = Umsatz × Multiple</t>
   </si>
   <si>
     <t xml:space="preserve">Ziel-Rendite (Multiple auf Einsatz)</t>
   </si>
   <si>
-    <t xml:space="preserve">Pre-Seed üblich 10–20x; Mittelwert 15x</t>
+    <t xml:space="preserve">Gründer-Annahme 10x = Untergrenze der Pre-Seed-üblichen 10–20x; konservativ Mittelwert 15x.</t>
   </si>
   <si>
     <t xml:space="preserve">Verwässerung durch spätere Runden (Seed, Series A, ESOP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Carta 2025: Median Seed ≈ 20 %, Series A ≈ 18 %; + ESOP ≈ 10 % → 1 − 0,8 × 0,82 × 0,9 ≈ 41 %; Annahme 45 %</t>
+    <t xml:space="preserve">Carta 2025: Seed ≈ 20 %, Series A ≈ 18 % → 1 − 0,8 × 0,82 ≈ 34 %; Gründer-Annahme 40 % (ohne vollen ESOP), konservativ 45 % (inkl. ESOP ≈ 10 %).</t>
   </si>
   <si>
     <t xml:space="preserve">Post-Money heute = Exit ÷ Ziel-Rendite × (1 − Verwässerung)</t>
@@ -1293,73 +1326,352 @@
     <t xml:space="preserve">Untergrenze 0</t>
   </si>
   <si>
-    <t xml:space="preserve">VC-Methode: Pre-Money bei Exit-Multiple (Zeilen) × Ziel-Rendite (Spalten)</t>
+    <t xml:space="preserve">VC-Methode (Umsatz J5 Basis, Verwässerung konservativ): Pre-Money bei Exit-Multiple (Zeilen) × Ziel-Rendite (Spalten)</t>
   </si>
   <si>
     <t xml:space="preserve">Multiple ↓ / Rendite →</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Ergebnis und Empfehlung</t>
+    <t xml:space="preserve">4. Referenzmethode (Investorensicht): Risk Factor Summation – nur Gründer-Sicht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basiswert = Scorecard-Referenz Gründer-Sicht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Methode (Ohio TechAngels/Payne): 12 Risiken, je −2 … +2, je Stufe ± 250.000 $ auf den regionalen Vergleichswert (eqvista; rho.co).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betrag je Stufe (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risikofaktor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Score (−2 … +2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zu-/Abschlag €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Begründung (Gründer-Sicht)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Management</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo-Gründer, erste Einstellung offen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entwicklungsstadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v2.1 ausgeliefert und in eigenen Streams im Einsatz; noch kein Umsatz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gesetzgebung / Politik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DSGVO/DSFA, Jugendschutz budgetiert; lokale Verarbeitung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Herstellung / Lieferkette</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reine Software, keine Lieferkette</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vertrieb / Marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">noch kein Vertrieb, keine Partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kapitalbeschaffung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Folgerunde (Seed) nötig – siehe Liquidität</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wettbewerb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kein direkter Sprach-Trigger-Wettbewerber; Nachbau durch Plattformen möglich</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Technologie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">funktionsfähig, 575+ Tests + e2e; Streaming-ASR &lt; 300 ms noch offen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rechtsstreit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GIF über KLIPY/GIPHY-API; Marke noch nicht eingetragen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">International</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DE/TR/EN von Beginn an, türkische Nische</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reputation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">neutral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exit-Potenzial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">strategische Käufer denkbar, aber unbelegt → neutral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summe Scores / Zu-/Abschlag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risk-Factor-Summation-Wert (Pre-Money)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Referenzmethoden (Investorensicht) – Zusammenfassung</t>
   </si>
   <si>
     <t xml:space="preserve">Methode</t>
   </si>
   <si>
+    <t xml:space="preserve">Gründer-Sicht €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Konservativ €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lesart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Berkus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gründer: 2×-Variante; konservativ: klassisch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scorecard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marktvergleich; Gründer-Referenz 2,5 Mio. €, konservativ 1,5 Mio. €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VC-Methode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gründer: optimistisches Szenario (Upside), Basis-Linie siehe unten; konservativ: Basis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risk Factor Summation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nur Gründer-Sicht (konservative Sicht nutzte drei Methoden)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spanne (Minimum)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spanne (Maximum)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gewichteter Mittelwert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gewichteter Mittelwert Gründer-Sicht mit VC-Basis-Linie statt optimistisch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zeigt, wie stark der Gründer-Mittelwert am optimistischen Szenario hängt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Konservativ: gewichteter Mittelwert auf 50 T€ gerundet (frühere Empfehlung, nur Referenz)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kontrolle: Gewichte je Sicht = 100 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Angebot der Gründer – max. 10 % für 250.000 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angebotener Anteil Investor:innen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vorgabe der Gründer: höchstens 10 % für 250.000 €.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Post-Money = Investition ÷ Anteil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-Money = Post-Money − Investition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anteil Gründer nach der Runde (ohne ESOP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kontrolle: Post-Money × Anteil = Investition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abstand zu den Referenzmethoden (transparent)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angebot Pre-Money ÷ gewichteter Mittelwert Gründer-Sicht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angebot Pre-Money − gewichteter Mittelwert Gründer-Sicht (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angebot Pre-Money ÷ Gründer-Mittelwert mit VC-Basis-Linie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angebot Pre-Money ÷ Minimum der Gründer-Spanne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angebot Pre-Money ÷ gewichteter Mittelwert konservativ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einordnung ggü. Gründer-Spanne (Formel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einordnung ggü. konservativer Investorensicht (Formel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lesart: Gegenüber der großzügigen, belegten Gründer-Sicht ist das Angebot zurückhaltend; gegenüber der konservativen Investorensicht ist es ambitioniert – Verhandlungsgrundlage sind die Argumente in Abschnitt 9.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Verhandlungsspanne – Anteil Investor:innen → Bewertung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anteil Investor:innen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Post-Money €</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pre-Money €</t>
   </si>
   <si>
-    <t xml:space="preserve">Warum dieses Gewicht</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Berkus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pre-revenue-Standard, Produktstand gut abbildbar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scorecard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marktvergleich DACH/TR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VC-Methode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hängt stark an 5-Jahres-Prognose ohne Umsatzhistorie → geringeres Gewicht</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spanne (Minimum)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spanne (Maximum)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gewichteter Mittelwert</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Empfohlene Pre-Money-Bewertung (auf 50 T€ gerundet)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Investition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Post-Money = Pre-Money + 250.000 €</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anteil Investor:innen (250.000 € ÷ Post-Money)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anteil Gründer nach der Runde (ohne ESOP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Alternative: Wandeldarlehen / SAFE (Vorschlag – mit Steuer-/Rechtsberater prüfen)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valuation Cap (Pre-Money) ≈ empfohlene Bewertung × Faktor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cap leicht über dem Preis der Eigenkapital-Variante, weil die Wandlung erst in der Seed-Runde erfolgt; Spanne 1,0–1,2 Mio. €.</t>
+    <t xml:space="preserve">Anteil Gründer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre ÷ Gründer-Mittel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre ÷ konservatives Mittel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">höhere Bewertung als das Angebot (Gründer-freundlich)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angebot der Gründer (Obergrenze laut Gründer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verhandlungskorridor bis hier: 10–12,5 % → Pre-Money 1,75–2,25 Mio. €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">außerhalb der Gründer-Vorgabe (nur Vergleich)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. Was müsste für 10× Investor-Rendite gelten? (Prüfung des Angebots)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Post-Money (Angebot der Gründer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verwässerung durch spätere Runden (Prüfannahme, Investorensicht)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bewusst die konservative Annahme (Carta + ESOP); mit Gründer-Annahme 40 % siehe Spalte E der Szenario-Tabelle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exit-Multiples auf den Umsatz J5 (Prüfwerte)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4x = konservativ (B2C-Abschlag), 6x = Gründer-Annahme (SaaS Capital 5,3x + Wachstumsaufschlag).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ziel-Rendite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nötiger Exit-Wert J5 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nötiger Umsatz J5 bei 4x €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nötiger Umsatz J5 bei 6x €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Getragen ab Szenario (4x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Getragen ab Szenario (6x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exit = Post-Money × Ziel-Rendite ÷ (1 − Verwässerung); Umsatz = Exit ÷ Multiple; Szenario = niedrigstes, dessen Umsatz J5 reicht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Szenario (GuV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umsatz J5 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implizite Rendite 4x (45 %)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implizite Rendite 6x (45 %)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implizite Rendite 6x (Gründer 40 %)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umsatz J5 ÷ Bedarf 10x @ 6x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ehrliche Lesart (Standardeingaben): Das Basis-Szenario trägt ≈ 4,2x (6x-Multiple) bzw. ≈ 2,8x (4x) – nicht 10x. 10x setzt das optimistische Szenario voraus: bei 6x und 45 % Verwässerung ≈ 9,8x (98 % des nötigen Umsatzes), bei 40 % Verwässerung ≈ 10,7x. 5x trägt das optimistische Szenario bei 4x und 6x.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9. Begründung / Argumente für das Angebot (10 % für 250.000 € → Pre-Money 2,25 Mio. €)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Funktionsfähiges Produkt v2.1 statt Konzept: Stimme → Effekt in Echtzeit, Leistungsmodus, sichere GIF-Suche; 575+ automatisierte Tests und eine e2e-Testsuite (Playwright) – das Technologierisiko ist weitgehend abgebaut.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Eigenes IP und eigene Inhalte: 238 Sprach-Trigger, 143 freie Sticker, Text- und Sticker-Inhalte sowie die Matcher-Logik sind selbst entwickelt; Markenanmeldung LiveFX (DE/EU/TR) ist budgetiert.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Drei Sprachen (DE/TR/EN) inkl. türkischer Nische: kaum spezialisierte Streaming-Tools auf Türkisch, eigene TR-Community als Startmarkt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vision-Optionen A–D auf derselben Engine: Erzählfilm/Story-Engine (A), WortBild Sprachenlernen (B), Räume/VR-AR (C), Studio/Auto-Edit (D) – Optionswert über das Creator-Tool hinaus.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Marktgröße: Live-Streaming-Markt 97–157 Mrd. USD, SAM 1–3 Mio. Creator (BP §6); Bildung/Sprachenlernen als zweiter Markt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Kapitaleffizienz: Produkt bis v2.1 ohne externes Kapital gebaut; die 250.000 € tragen laut Modell 18 Monate bis Gate 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vision-Trailer und Prototypen (Erzählfilm, WortBild als lauffähige HTML-Prototypen; 30-s-Produkttrailer) machen die Linien sichtbar – Investor:innen sehen mehr als eine Folie.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ehrlich dagegen: Solo-Gründer, noch kein Umsatz und keine Partner; konservative Methoden ergeben 0,2–1,4 Mio. € Pre-Money.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10. Alternative: Wandeldarlehen / SAFE (Vorschlag – mit Steuer-/Rechtsberater prüfen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valuation Cap (Pre-Money)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cap = Pre-Money des Gründer-Angebots (2,25 Mio. €) → Anteil am Cap ≈ 10 %.</t>
   </si>
   <si>
     <t xml:space="preserve">Discount auf den Preis der Folgerunde</t>
@@ -1383,12 +1695,18 @@
     <t xml:space="preserve">Wandlungsbewertung = MIN(Cap; Seed-Pre × (1 − Discount))</t>
   </si>
   <si>
-    <t xml:space="preserve">Anteil bei Wandlung (vereinfacht, vor Seed-Geld)</t>
+    <t xml:space="preserve">Anteil bei Wandlung im Beispiel (vereinfacht, vor Seed-Geld)</t>
   </si>
   <si>
     <t xml:space="preserve">Max. Anteil am Cap ohne Zins (250.000 ÷ (Cap + 250.000))</t>
   </si>
   <si>
+    <t xml:space="preserve">Max. Anteil am Cap mit Zins (Wandlungsbetrag ÷ (Cap + Wandlungsbetrag))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mit 5 % Zins über 18 Monate liegt der Anteil leicht über 10 % – ggf. Zins niedriger oder Cap entsprechend höher verhandeln.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Alle Bewertungen: Vorschlag – mit Steuer-/Rechtsberater prüfen. Keine Anlageberatung.</t>
   </si>
   <si>
@@ -1758,13 +2076,55 @@
     <t xml:space="preserve">Post-money valuation</t>
   </si>
   <si>
-    <t xml:space="preserve">Anteil Investor:innen</t>
-  </si>
-  <si>
     <t xml:space="preserve">Yatırımcı payı</t>
   </si>
   <si>
     <t xml:space="preserve">Investor stake</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angebot der Gründer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kurucuların teklifi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Founders' offer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referenzmethoden (Investorensicht)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referans yöntemler (yatırımcı bakışı)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference methods (investor view)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gründer-Sicht / konservative Sicht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kurucu bakışı / temkinli bakış</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Founder view / conservative view</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verhandlungsspanne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pazarlık aralığı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Negotiation range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Begründung / Argumente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gerekçe / argümanlar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rationale / arguments</t>
   </si>
   <si>
     <t xml:space="preserve">Wandeldarlehen / SAFE, Valuation Cap, Discount</t>
@@ -1804,7 +2164,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="13">
+  <numFmts count="15">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0&quot; €&quot;;\(#,##0&quot; €)&quot;;\–"/>
     <numFmt numFmtId="166" formatCode="0.0%;\(0.0%\);\–"/>
@@ -1815,9 +2175,11 @@
     <numFmt numFmtId="171" formatCode="0.0;\(0.0\);\–"/>
     <numFmt numFmtId="172" formatCode="0.000"/>
     <numFmt numFmtId="173" formatCode="0.0\x"/>
-    <numFmt numFmtId="174" formatCode="0.00\x"/>
-    <numFmt numFmtId="175" formatCode="\+0.0%;\-0.0%;0.0%"/>
-    <numFmt numFmtId="176" formatCode="#,##0"/>
+    <numFmt numFmtId="174" formatCode="\+0;\-0;0"/>
+    <numFmt numFmtId="175" formatCode="\+#,##0&quot; €&quot;;\-#,##0&quot; €&quot;;&quot;0 €&quot;"/>
+    <numFmt numFmtId="176" formatCode="0.00\x"/>
+    <numFmt numFmtId="177" formatCode="\+0.0%;\-0.0%;0.0%"/>
+    <numFmt numFmtId="178" formatCode="#,##0"/>
   </numFmts>
   <fonts count="17">
     <font>
@@ -2010,7 +2372,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="55">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2187,11 +2549,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="174" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="175" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="176" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="176" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2199,11 +2581,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="177" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2518,11 +2904,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="85082835"/>
-        <c:axId val="92090136"/>
+        <c:axId val="75436296"/>
+        <c:axId val="33811507"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="85082835"/>
+        <c:axId val="75436296"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2554,7 +2940,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92090136"/>
+        <c:crossAx val="33811507"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2562,7 +2948,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="92090136"/>
+        <c:axId val="33811507"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2638,7 +3024,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85082835"/>
+        <c:crossAx val="75436296"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3606,11 +3992,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="62108771"/>
-        <c:axId val="59110876"/>
+        <c:axId val="17868832"/>
+        <c:axId val="11820272"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="62108771"/>
+        <c:axId val="17868832"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3676,7 +4062,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59110876"/>
+        <c:crossAx val="11820272"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3684,7 +4070,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="59110876"/>
+        <c:axId val="11820272"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3760,7 +4146,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62108771"/>
+        <c:crossAx val="17868832"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -17871,12 +18257,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="95"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17902,7 +18288,9 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
+      <c r="A3" s="3" t="s">
+        <v>366</v>
+      </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -17911,92 +18299,73 @@
       <c r="G3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>366</v>
-      </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" s="12" t="s">
+      <c r="A5" s="4" t="s">
         <v>367</v>
       </c>
-      <c r="C5" s="12" t="s">
-        <v>368</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>369</v>
-      </c>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12" t="s">
-        <v>370</v>
-      </c>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>371</v>
-      </c>
-      <c r="B6" s="8" t="n">
-        <v>500000</v>
-      </c>
-      <c r="C6" s="40" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D6" s="15" t="n">
-        <f aca="false">B6*C6</f>
-        <v>300000</v>
-      </c>
+        <v>368</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
-      <c r="G6" s="6" t="s">
-        <v>372</v>
+      <c r="G6" s="3" t="s">
+        <v>369</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>500000</v>
       </c>
-      <c r="C7" s="40" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="D7" s="15" t="n">
-        <f aca="false">B7*C7</f>
-        <v>350000</v>
-      </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="3" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>373</v>
+      </c>
+      <c r="D8" s="12" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+      <c r="E8" s="12" t="s">
         <v>375</v>
       </c>
-      <c r="B8" s="8" t="n">
-        <v>500000</v>
-      </c>
-      <c r="C8" s="40" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D8" s="15" t="n">
-        <f aca="false">B8*C8</f>
-        <v>150000</v>
-      </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="6" t="s">
+      <c r="F8" s="12"/>
+      <c r="G8" s="12" t="s">
         <v>376</v>
       </c>
     </row>
@@ -18004,17 +18373,20 @@
       <c r="A9" s="6" t="s">
         <v>377</v>
       </c>
-      <c r="B9" s="8" t="n">
-        <v>500000</v>
-      </c>
-      <c r="C9" s="40" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D9" s="15" t="n">
-        <f aca="false">B9*C9</f>
-        <v>50000</v>
-      </c>
-      <c r="E9" s="2"/>
+      <c r="B9" s="40" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C9" s="21" t="n">
+        <f aca="false">Bewertung!$B$6*B9</f>
+        <v>700000</v>
+      </c>
+      <c r="D9" s="40" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <f aca="false">Bewertung!$B$7*D9</f>
+        <v>300000</v>
+      </c>
       <c r="F9" s="2"/>
       <c r="G9" s="6" t="s">
         <v>378</v>
@@ -18024,173 +18396,182 @@
       <c r="A10" s="6" t="s">
         <v>379</v>
       </c>
-      <c r="B10" s="8" t="n">
-        <v>500000</v>
-      </c>
-      <c r="C10" s="40" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D10" s="15" t="n">
-        <f aca="false">B10*C10</f>
-        <v>50000</v>
-      </c>
-      <c r="E10" s="2"/>
+      <c r="B10" s="40" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C10" s="21" t="n">
+        <f aca="false">Bewertung!$B$6*B10</f>
+        <v>800000</v>
+      </c>
+      <c r="D10" s="40" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <f aca="false">Bewertung!$B$7*D10</f>
+        <v>350000</v>
+      </c>
       <c r="F10" s="2"/>
       <c r="G10" s="6" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="6" t="s">
         <v>381</v>
       </c>
-      <c r="B11" s="15" t="n">
-        <f aca="false">SUM(B6:B10)</f>
-        <v>2500000</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="24" t="n">
-        <f aca="false">SUM(D6:D10)</f>
+      <c r="B11" s="40" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C11" s="21" t="n">
+        <f aca="false">Bewertung!$B$6*B11</f>
+        <v>500000</v>
+      </c>
+      <c r="D11" s="40" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <f aca="false">Bewertung!$B$7*D11</f>
+        <v>150000</v>
+      </c>
+      <c r="F11" s="2"/>
+      <c r="G11" s="6" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="B12" s="40" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C12" s="21" t="n">
+        <f aca="false">Bewertung!$B$6*B12</f>
+        <v>250000</v>
+      </c>
+      <c r="D12" s="40" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <f aca="false">Bewertung!$B$7*D12</f>
+        <v>50000</v>
+      </c>
+      <c r="F12" s="2"/>
+      <c r="G12" s="6" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="B13" s="40" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C13" s="21" t="n">
+        <f aca="false">Bewertung!$B$6*B13</f>
+        <v>100000</v>
+      </c>
+      <c r="D13" s="40" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <f aca="false">Bewertung!$B$7*D13</f>
+        <v>50000</v>
+      </c>
+      <c r="F13" s="2"/>
+      <c r="G13" s="6" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="16" t="s">
+        <v>387</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="24" t="n">
+        <f aca="false">SUM(C9:C13)</f>
+        <v>2350000</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="17" t="n">
+        <f aca="false">SUM(E9:E13)</f>
         <v>900000</v>
       </c>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="3" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>383</v>
-      </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>384</v>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
       <c r="F14" s="2"/>
-      <c r="G14" s="3" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>386</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>387</v>
-      </c>
-      <c r="D15" s="12" t="s">
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>388</v>
       </c>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>390</v>
-      </c>
-      <c r="B16" s="9" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C16" s="9" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D16" s="41" t="n">
-        <f aca="false">B16*C16</f>
-        <v>0.18</v>
-      </c>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="6" t="s">
-        <v>391</v>
-      </c>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>392</v>
-      </c>
-      <c r="B17" s="9" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="C17" s="9" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="D17" s="41" t="n">
-        <f aca="false">B17*C17</f>
-        <v>0.3125</v>
-      </c>
+        <v>389</v>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
-      <c r="G17" s="6" t="s">
-        <v>393</v>
+      <c r="G17" s="3" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>394</v>
-      </c>
-      <c r="B18" s="9" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C18" s="9" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="D18" s="41" t="n">
-        <f aca="false">B18*C18</f>
-        <v>0.18</v>
-      </c>
+        <v>391</v>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
-      <c r="G18" s="6" t="s">
+      <c r="G18" s="3" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>394</v>
+      </c>
+      <c r="D19" s="12" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
+      <c r="E19" s="12" t="s">
         <v>396</v>
       </c>
-      <c r="B19" s="9" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C19" s="9" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="D19" s="41" t="n">
-        <f aca="false">B19*C19</f>
-        <v>0.09</v>
-      </c>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="6" t="s">
+      <c r="F19" s="12" t="s">
         <v>397</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>376</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18198,17 +18579,22 @@
         <v>398</v>
       </c>
       <c r="B20" s="9" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="D20" s="41" t="n">
         <f aca="false">B20*C20</f>
-        <v>0.07</v>
-      </c>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
+        <v>0.3</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F20" s="41" t="n">
+        <f aca="false">B20*E20</f>
+        <v>0.18</v>
+      </c>
       <c r="G20" s="6" t="s">
         <v>399</v>
       </c>
@@ -18218,17 +18604,22 @@
         <v>400</v>
       </c>
       <c r="B21" s="9" t="n">
-        <v>0.05</v>
+        <v>0.25</v>
       </c>
       <c r="C21" s="9" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="D21" s="41" t="n">
         <f aca="false">B21*C21</f>
-        <v>0.05</v>
-      </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
+        <v>0.35</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F21" s="41" t="n">
+        <f aca="false">B21*E21</f>
+        <v>0.3125</v>
+      </c>
       <c r="G21" s="6" t="s">
         <v>401</v>
       </c>
@@ -18238,17 +18629,22 @@
         <v>402</v>
       </c>
       <c r="B22" s="9" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="D22" s="41" t="n">
         <f aca="false">B22*C22</f>
-        <v>0.055</v>
-      </c>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
+        <v>0.21</v>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F22" s="41" t="n">
+        <f aca="false">B22*E22</f>
+        <v>0.18</v>
+      </c>
       <c r="G22" s="6" t="s">
         <v>403</v>
       </c>
@@ -18257,417 +18653,498 @@
       <c r="A23" s="6" t="s">
         <v>404</v>
       </c>
-      <c r="B23" s="25" t="n">
-        <f aca="false">SUM(B16:B22)</f>
+      <c r="B23" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D23" s="41" t="n">
+        <f aca="false">B23*C23</f>
+        <v>0.13</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F23" s="41" t="n">
+        <f aca="false">B23*E23</f>
+        <v>0.09</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
+        <v>406</v>
+      </c>
+      <c r="B24" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C24" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D24" s="41" t="n">
+        <f aca="false">B24*C24</f>
+        <v>0.08</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F24" s="41" t="n">
+        <f aca="false">B24*E24</f>
+        <v>0.07</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="B25" s="9" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C25" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="41" t="n">
-        <f aca="false">SUM(D16:D22)</f>
-        <v>0.9375</v>
-      </c>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="16" t="s">
-        <v>405</v>
-      </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="42" t="n">
-        <f aca="false">Bewertung!$B$14*D23</f>
-        <v>1406250</v>
-      </c>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
+      <c r="D25" s="41" t="n">
+        <f aca="false">B25*C25</f>
+        <v>0.05</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="41" t="n">
+        <f aca="false">B25*E25</f>
+        <v>0.05</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>409</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
-        <v>406</v>
-      </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
+      <c r="A26" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="B26" s="9" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D26" s="41" t="n">
+        <f aca="false">B26*C26</f>
+        <v>0.06</v>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F26" s="41" t="n">
+        <f aca="false">B26*E26</f>
+        <v>0.055</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>411</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>407</v>
-      </c>
-      <c r="B27" s="21" t="n">
-        <f aca="false">'GuV 5 Jahre'!$G$36</f>
-        <v>3151812.5</v>
+        <v>412</v>
+      </c>
+      <c r="B27" s="25" t="n">
+        <f aca="false">SUM(B20:B26)</f>
+        <v>1</v>
       </c>
       <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
+      <c r="D27" s="41" t="n">
+        <f aca="false">SUM(D20:D26)</f>
+        <v>1.18</v>
+      </c>
       <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="3" t="s">
-        <v>408</v>
-      </c>
+      <c r="F27" s="41" t="n">
+        <f aca="false">SUM(F20:F26)</f>
+        <v>0.9375</v>
+      </c>
+      <c r="G27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
-        <v>409</v>
-      </c>
-      <c r="B28" s="43" t="n">
-        <v>4</v>
-      </c>
+      <c r="A28" s="16" t="s">
+        <v>413</v>
+      </c>
+      <c r="B28" s="2"/>
       <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
+      <c r="D28" s="42" t="n">
+        <f aca="false">Bewertung!$B$17*D27</f>
+        <v>2950000</v>
+      </c>
       <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="3" t="s">
-        <v>410</v>
-      </c>
+      <c r="F28" s="23" t="n">
+        <f aca="false">Bewertung!$B$18*F27</f>
+        <v>1406250</v>
+      </c>
+      <c r="G28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
-        <v>411</v>
-      </c>
-      <c r="B29" s="15" t="n">
-        <f aca="false">B27*B28</f>
-        <v>12607250</v>
-      </c>
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
-      <c r="G29" s="3" t="s">
-        <v>412</v>
-      </c>
+      <c r="G29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
-        <v>413</v>
-      </c>
-      <c r="B30" s="43" t="n">
-        <v>15</v>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="3" t="s">
+      <c r="A30" s="4" t="s">
         <v>414</v>
       </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
+      <c r="B30" s="5"/>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+    </row>
+    <row r="31" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="B31" s="12" t="s">
         <v>415</v>
       </c>
-      <c r="B31" s="9" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="3" t="s">
+      <c r="C31" s="12" t="s">
         <v>416</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>417</v>
+      </c>
+      <c r="E31" s="12"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="12" t="s">
+        <v>418</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>417</v>
-      </c>
-      <c r="B32" s="15" t="n">
-        <f aca="false">B29/B30*(1-B31)</f>
-        <v>462265.833333333</v>
-      </c>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
+        <v>419</v>
+      </c>
+      <c r="B32" s="21" t="n">
+        <f aca="false">'GuV 5 Jahre'!$G$57</f>
+        <v>7444105</v>
+      </c>
+      <c r="C32" s="21" t="n">
+        <f aca="false">'GuV 5 Jahre'!$G$36</f>
+        <v>3151812.5</v>
+      </c>
+      <c r="D32" s="21" t="n">
+        <f aca="false">'GuV 5 Jahre'!$G$36</f>
+        <v>3151812.5</v>
+      </c>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
-      <c r="G32" s="3"/>
+      <c r="G32" s="3" t="s">
+        <v>420</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>418</v>
-      </c>
-      <c r="B33" s="21" t="n">
+        <v>421</v>
+      </c>
+      <c r="B33" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="C33" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="D33" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="3" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="B34" s="15" t="n">
+        <f aca="false">B32*B33</f>
+        <v>44664630</v>
+      </c>
+      <c r="C34" s="15" t="n">
+        <f aca="false">C32*C33</f>
+        <v>18910875</v>
+      </c>
+      <c r="D34" s="15" t="n">
+        <f aca="false">D32*D33</f>
+        <v>12607250</v>
+      </c>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="3"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="s">
+        <v>424</v>
+      </c>
+      <c r="B35" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="C35" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="D35" s="43" t="n">
+        <v>15</v>
+      </c>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="3" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="B36" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C36" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D36" s="9" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="3" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>428</v>
+      </c>
+      <c r="B37" s="15" t="n">
+        <f aca="false">B34/B35*(1-B36)</f>
+        <v>2679877.8</v>
+      </c>
+      <c r="C37" s="15" t="n">
+        <f aca="false">C34/C35*(1-C36)</f>
+        <v>1134652.5</v>
+      </c>
+      <c r="D37" s="15" t="n">
+        <f aca="false">D34/D35*(1-D36)</f>
+        <v>462265.833333333</v>
+      </c>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="3"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="B38" s="21" t="n">
         <f aca="false">Annahmen!$B$6</f>
         <v>250000</v>
       </c>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="3"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="16" t="s">
-        <v>419</v>
-      </c>
-      <c r="B34" s="24" t="n">
-        <f aca="false">MAX(0,B32-B33)</f>
-        <v>212265.833333333</v>
-      </c>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="3" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="34" t="s">
-        <v>421</v>
-      </c>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
-        <v>422</v>
-      </c>
-      <c r="B37" s="43" t="n">
-        <v>10</v>
-      </c>
-      <c r="C37" s="43" t="n">
-        <v>15</v>
-      </c>
-      <c r="D37" s="43" t="n">
-        <v>20</v>
-      </c>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="43" t="n">
-        <v>3</v>
-      </c>
-      <c r="B38" s="21" t="n">
-        <f aca="false">MAX(0,Bewertung!$B$27*$A38/B$37*(1-Bewertung!$B$31)-Bewertung!$B$33)</f>
-        <v>270049.0625</v>
-      </c>
       <c r="C38" s="21" t="n">
-        <f aca="false">MAX(0,Bewertung!$B$27*$A38/C$37*(1-Bewertung!$B$31)-Bewertung!$B$33)</f>
-        <v>96699.375</v>
+        <f aca="false">Annahmen!$B$6</f>
+        <v>250000</v>
       </c>
       <c r="D38" s="21" t="n">
-        <f aca="false">MAX(0,Bewertung!$B$27*$A38/D$37*(1-Bewertung!$B$31)-Bewertung!$B$33)</f>
-        <v>10024.53125</v>
+        <f aca="false">Annahmen!$B$6</f>
+        <v>250000</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
+      <c r="G38" s="3"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="43" t="n">
-        <v>4</v>
-      </c>
-      <c r="B39" s="21" t="n">
-        <f aca="false">MAX(0,Bewertung!$B$27*$A39/B$37*(1-Bewertung!$B$31)-Bewertung!$B$33)</f>
-        <v>443398.75</v>
-      </c>
-      <c r="C39" s="21" t="n">
-        <f aca="false">MAX(0,Bewertung!$B$27*$A39/C$37*(1-Bewertung!$B$31)-Bewertung!$B$33)</f>
+      <c r="A39" s="16" t="s">
+        <v>430</v>
+      </c>
+      <c r="B39" s="24" t="n">
+        <f aca="false">MAX(0,B37-B38)</f>
+        <v>2429877.8</v>
+      </c>
+      <c r="C39" s="17" t="n">
+        <f aca="false">MAX(0,C37-C38)</f>
+        <v>884652.5</v>
+      </c>
+      <c r="D39" s="17" t="n">
+        <f aca="false">MAX(0,D37-D38)</f>
         <v>212265.833333333</v>
-      </c>
-      <c r="D39" s="21" t="n">
-        <f aca="false">MAX(0,Bewertung!$B$27*$A39/D$37*(1-Bewertung!$B$31)-Bewertung!$B$33)</f>
-        <v>96699.375</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
+      <c r="G39" s="3" t="s">
+        <v>431</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="43" t="n">
-        <v>5</v>
-      </c>
-      <c r="B40" s="21" t="n">
-        <f aca="false">MAX(0,Bewertung!$B$27*$A40/B$37*(1-Bewertung!$B$31)-Bewertung!$B$33)</f>
-        <v>616748.4375</v>
-      </c>
-      <c r="C40" s="21" t="n">
-        <f aca="false">MAX(0,Bewertung!$B$27*$A40/C$37*(1-Bewertung!$B$31)-Bewertung!$B$33)</f>
-        <v>327832.291666667</v>
-      </c>
-      <c r="D40" s="21" t="n">
-        <f aca="false">MAX(0,Bewertung!$B$27*$A40/D$37*(1-Bewertung!$B$31)-Bewertung!$B$33)</f>
-        <v>183374.21875</v>
-      </c>
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
       <c r="E40" s="2"/>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="43" t="n">
-        <v>6</v>
-      </c>
-      <c r="B41" s="21" t="n">
-        <f aca="false">MAX(0,Bewertung!$B$27*$A41/B$37*(1-Bewertung!$B$31)-Bewertung!$B$33)</f>
-        <v>790098.125</v>
-      </c>
-      <c r="C41" s="21" t="n">
-        <f aca="false">MAX(0,Bewertung!$B$27*$A41/C$37*(1-Bewertung!$B$31)-Bewertung!$B$33)</f>
-        <v>443398.75</v>
-      </c>
-      <c r="D41" s="21" t="n">
-        <f aca="false">MAX(0,Bewertung!$B$27*$A41/D$37*(1-Bewertung!$B$31)-Bewertung!$B$33)</f>
-        <v>270049.0625</v>
-      </c>
+      <c r="A41" s="34" t="s">
+        <v>432</v>
+      </c>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
       <c r="E41" s="2"/>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="2"/>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
+      <c r="A42" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="B42" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="C42" s="43" t="n">
+        <v>15</v>
+      </c>
+      <c r="D42" s="43" t="n">
+        <v>20</v>
+      </c>
       <c r="E42" s="2"/>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
-        <v>423</v>
-      </c>
-      <c r="B43" s="5"/>
-      <c r="C43" s="5"/>
-      <c r="D43" s="5"/>
-      <c r="E43" s="5"/>
-      <c r="F43" s="5"/>
-      <c r="G43" s="5"/>
+      <c r="A43" s="43" t="n">
+        <v>3</v>
+      </c>
+      <c r="B43" s="21" t="n">
+        <f aca="false">MAX(0,Bewertung!$D$32*$A43/B$42*(1-Bewertung!$D$36)-Bewertung!$D$38)</f>
+        <v>270049.0625</v>
+      </c>
+      <c r="C43" s="21" t="n">
+        <f aca="false">MAX(0,Bewertung!$D$32*$A43/C$42*(1-Bewertung!$D$36)-Bewertung!$D$38)</f>
+        <v>96699.375</v>
+      </c>
+      <c r="D43" s="21" t="n">
+        <f aca="false">MAX(0,Bewertung!$D$32*$A43/D$42*(1-Bewertung!$D$36)-Bewertung!$D$38)</f>
+        <v>10024.53125</v>
+      </c>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="12" t="s">
-        <v>424</v>
-      </c>
-      <c r="B44" s="12" t="s">
-        <v>425</v>
-      </c>
-      <c r="C44" s="12" t="s">
-        <v>386</v>
-      </c>
-      <c r="D44" s="12"/>
-      <c r="E44" s="12"/>
-      <c r="F44" s="12"/>
-      <c r="G44" s="12" t="s">
-        <v>426</v>
-      </c>
+      <c r="A44" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="B44" s="21" t="n">
+        <f aca="false">MAX(0,Bewertung!$D$32*$A44/B$42*(1-Bewertung!$D$36)-Bewertung!$D$38)</f>
+        <v>443398.75</v>
+      </c>
+      <c r="C44" s="21" t="n">
+        <f aca="false">MAX(0,Bewertung!$D$32*$A44/C$42*(1-Bewertung!$D$36)-Bewertung!$D$38)</f>
+        <v>212265.833333333</v>
+      </c>
+      <c r="D44" s="21" t="n">
+        <f aca="false">MAX(0,Bewertung!$D$32*$A44/D$42*(1-Bewertung!$D$36)-Bewertung!$D$38)</f>
+        <v>96699.375</v>
+      </c>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="6" t="s">
-        <v>427</v>
+      <c r="A45" s="43" t="n">
+        <v>5</v>
       </c>
       <c r="B45" s="21" t="n">
-        <f aca="false">Bewertung!$D$11</f>
-        <v>900000</v>
-      </c>
-      <c r="C45" s="9" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D45" s="2"/>
+        <f aca="false">MAX(0,Bewertung!$D$32*$A45/B$42*(1-Bewertung!$D$36)-Bewertung!$D$38)</f>
+        <v>616748.4375</v>
+      </c>
+      <c r="C45" s="21" t="n">
+        <f aca="false">MAX(0,Bewertung!$D$32*$A45/C$42*(1-Bewertung!$D$36)-Bewertung!$D$38)</f>
+        <v>327832.291666667</v>
+      </c>
+      <c r="D45" s="21" t="n">
+        <f aca="false">MAX(0,Bewertung!$D$32*$A45/D$42*(1-Bewertung!$D$36)-Bewertung!$D$38)</f>
+        <v>183374.21875</v>
+      </c>
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
-      <c r="G45" s="6" t="s">
-        <v>428</v>
-      </c>
+      <c r="G45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="6" t="s">
-        <v>429</v>
+      <c r="A46" s="43" t="n">
+        <v>6</v>
       </c>
       <c r="B46" s="21" t="n">
-        <f aca="false">Bewertung!$D$24</f>
-        <v>1406250</v>
-      </c>
-      <c r="C46" s="9" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D46" s="2"/>
+        <f aca="false">MAX(0,Bewertung!$D$32*$A46/B$42*(1-Bewertung!$D$36)-Bewertung!$D$38)</f>
+        <v>790098.125</v>
+      </c>
+      <c r="C46" s="21" t="n">
+        <f aca="false">MAX(0,Bewertung!$D$32*$A46/C$42*(1-Bewertung!$D$36)-Bewertung!$D$38)</f>
+        <v>443398.75</v>
+      </c>
+      <c r="D46" s="21" t="n">
+        <f aca="false">MAX(0,Bewertung!$D$32*$A46/D$42*(1-Bewertung!$D$36)-Bewertung!$D$38)</f>
+        <v>270049.0625</v>
+      </c>
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
-      <c r="G46" s="6" t="s">
-        <v>430</v>
-      </c>
+      <c r="G46" s="2"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="6" t="s">
-        <v>431</v>
-      </c>
-      <c r="B47" s="21" t="n">
-        <f aca="false">Bewertung!$B$34</f>
-        <v>212265.833333333</v>
-      </c>
-      <c r="C47" s="9" t="n">
-        <v>0.2</v>
-      </c>
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
       <c r="F47" s="2"/>
-      <c r="G47" s="6" t="s">
-        <v>432</v>
-      </c>
+      <c r="G47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="6" t="s">
-        <v>433</v>
-      </c>
-      <c r="B48" s="15" t="n">
-        <f aca="false">MIN(B45:B47)</f>
-        <v>212265.833333333</v>
-      </c>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
-      <c r="F48" s="2"/>
-      <c r="G48" s="2"/>
+      <c r="A48" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>434</v>
-      </c>
-      <c r="B49" s="15" t="n">
-        <f aca="false">MAX(B45:B47)</f>
-        <v>1406250</v>
+        <v>435</v>
+      </c>
+      <c r="B49" s="21" t="n">
+        <f aca="false">Bewertung!$B$17</f>
+        <v>2500000</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
-      <c r="G49" s="2"/>
+      <c r="G49" s="3" t="s">
+        <v>436</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="B50" s="15" t="n">
-        <f aca="false">SUMPRODUCT(B45:B47,C45:C47)/SUM(C45:C47)</f>
-        <v>964953.166666667</v>
+        <v>437</v>
+      </c>
+      <c r="B50" s="8" t="n">
+        <v>250000</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
@@ -18676,190 +19153,250 @@
       <c r="G50" s="2"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="16" t="s">
-        <v>436</v>
-      </c>
-      <c r="B51" s="42" t="n">
-        <f aca="false">ROUND(Bewertung!$B$50/50000,0)*50000</f>
-        <v>950000</v>
-      </c>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="2"/>
+      <c r="A51" s="12" t="s">
+        <v>438</v>
+      </c>
+      <c r="B51" s="12" t="s">
+        <v>439</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>440</v>
+      </c>
+      <c r="D51" s="12"/>
+      <c r="E51" s="12"/>
+      <c r="F51" s="12"/>
+      <c r="G51" s="12" t="s">
+        <v>441</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>437</v>
-      </c>
-      <c r="B52" s="21" t="n">
-        <f aca="false">Annahmen!$B$6</f>
-        <v>250000</v>
-      </c>
-      <c r="C52" s="2"/>
+        <v>442</v>
+      </c>
+      <c r="B52" s="44" t="n">
+        <v>-1</v>
+      </c>
+      <c r="C52" s="45" t="n">
+        <f aca="false">B52*Bewertung!$B$50</f>
+        <v>-250000</v>
+      </c>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
       <c r="F52" s="2"/>
-      <c r="G52" s="2"/>
+      <c r="G52" s="6" t="s">
+        <v>443</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="16" t="s">
-        <v>438</v>
-      </c>
-      <c r="B53" s="23" t="n">
-        <f aca="false">Bewertung!$B$51+Annahmen!$B$6</f>
-        <v>1200000</v>
-      </c>
-      <c r="C53" s="2"/>
+      <c r="A53" s="6" t="s">
+        <v>444</v>
+      </c>
+      <c r="B53" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" s="45" t="n">
+        <f aca="false">B53*Bewertung!$B$50</f>
+        <v>250000</v>
+      </c>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
       <c r="F53" s="2"/>
-      <c r="G53" s="2"/>
+      <c r="G53" s="6" t="s">
+        <v>445</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="16" t="s">
-        <v>439</v>
+      <c r="A54" s="6" t="s">
+        <v>446</v>
       </c>
       <c r="B54" s="44" t="n">
-        <f aca="false">Annahmen!$B$6/Bewertung!$B$53</f>
-        <v>0.208333333333333</v>
-      </c>
-      <c r="C54" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="C54" s="45" t="n">
+        <f aca="false">B54*Bewertung!$B$50</f>
+        <v>0</v>
+      </c>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
-      <c r="G54" s="2"/>
+      <c r="G54" s="6" t="s">
+        <v>447</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="s">
-        <v>440</v>
-      </c>
-      <c r="B55" s="19" t="n">
-        <f aca="false">1-Bewertung!$B$54</f>
-        <v>0.791666666666667</v>
-      </c>
-      <c r="C55" s="2"/>
+        <v>448</v>
+      </c>
+      <c r="B55" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" s="45" t="n">
+        <f aca="false">B55*Bewertung!$B$50</f>
+        <v>250000</v>
+      </c>
       <c r="D55" s="2"/>
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
-      <c r="G55" s="2"/>
+      <c r="G55" s="6" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
+      <c r="A56" s="6" t="s">
+        <v>450</v>
+      </c>
+      <c r="B56" s="44" t="n">
+        <v>-1</v>
+      </c>
+      <c r="C56" s="45" t="n">
+        <f aca="false">B56*Bewertung!$B$50</f>
+        <v>-250000</v>
+      </c>
       <c r="D56" s="2"/>
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
-      <c r="G56" s="2"/>
+      <c r="G56" s="6" t="s">
+        <v>451</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="4" t="s">
-        <v>441</v>
-      </c>
-      <c r="B57" s="5"/>
-      <c r="C57" s="5"/>
-      <c r="D57" s="5"/>
-      <c r="E57" s="5"/>
-      <c r="F57" s="5"/>
-      <c r="G57" s="5"/>
+      <c r="A57" s="6" t="s">
+        <v>452</v>
+      </c>
+      <c r="B57" s="44" t="n">
+        <v>-1</v>
+      </c>
+      <c r="C57" s="45" t="n">
+        <f aca="false">B57*Bewertung!$B$50</f>
+        <v>-250000</v>
+      </c>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="6" t="s">
+        <v>453</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="s">
-        <v>442</v>
-      </c>
-      <c r="B58" s="39" t="n">
-        <f aca="false">ROUND(Bewertung!$B$51*C58/50000,0)*50000</f>
-        <v>1150000</v>
+        <v>454</v>
+      </c>
+      <c r="B58" s="44" t="n">
+        <v>1</v>
       </c>
       <c r="C58" s="45" t="n">
-        <v>1.2</v>
+        <f aca="false">B58*Bewertung!$B$50</f>
+        <v>250000</v>
       </c>
       <c r="D58" s="2"/>
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
-      <c r="G58" s="3" t="s">
-        <v>443</v>
+      <c r="G58" s="6" t="s">
+        <v>455</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="6" t="s">
-        <v>444</v>
-      </c>
-      <c r="B59" s="9" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C59" s="2"/>
+        <v>456</v>
+      </c>
+      <c r="B59" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" s="45" t="n">
+        <f aca="false">B59*Bewertung!$B$50</f>
+        <v>250000</v>
+      </c>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
       <c r="F59" s="2"/>
-      <c r="G59" s="3" t="s">
-        <v>445</v>
+      <c r="G59" s="6" t="s">
+        <v>457</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="6" t="s">
-        <v>446</v>
-      </c>
-      <c r="B60" s="9" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="C60" s="2"/>
+        <v>458</v>
+      </c>
+      <c r="B60" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C60" s="45" t="n">
+        <f aca="false">B60*Bewertung!$B$50</f>
+        <v>0</v>
+      </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
-      <c r="G60" s="2"/>
+      <c r="G60" s="6" t="s">
+        <v>459</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="6" t="s">
-        <v>447</v>
-      </c>
-      <c r="B61" s="10" t="n">
-        <v>18</v>
-      </c>
-      <c r="C61" s="2"/>
+        <v>460</v>
+      </c>
+      <c r="B61" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" s="45" t="n">
+        <f aca="false">B61*Bewertung!$B$50</f>
+        <v>250000</v>
+      </c>
       <c r="D61" s="2"/>
       <c r="E61" s="2"/>
       <c r="F61" s="2"/>
-      <c r="G61" s="2"/>
+      <c r="G61" s="6" t="s">
+        <v>461</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="6" t="s">
-        <v>448</v>
-      </c>
-      <c r="B62" s="21" t="n">
-        <f aca="false">Annahmen!$B$6*(1+Bewertung!$B$60*Bewertung!$B$61/12)</f>
-        <v>268750</v>
-      </c>
-      <c r="C62" s="2"/>
+        <v>462</v>
+      </c>
+      <c r="B62" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C62" s="45" t="n">
+        <f aca="false">B62*Bewertung!$B$50</f>
+        <v>0</v>
+      </c>
       <c r="D62" s="2"/>
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
-      <c r="G62" s="2"/>
+      <c r="G62" s="6" t="s">
+        <v>463</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="6" t="s">
-        <v>449</v>
-      </c>
-      <c r="B63" s="8" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="C63" s="2"/>
+        <v>464</v>
+      </c>
+      <c r="B63" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C63" s="45" t="n">
+        <f aca="false">B63*Bewertung!$B$50</f>
+        <v>0</v>
+      </c>
       <c r="D63" s="2"/>
       <c r="E63" s="2"/>
       <c r="F63" s="2"/>
-      <c r="G63" s="2"/>
+      <c r="G63" s="6" t="s">
+        <v>465</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="6" t="s">
-        <v>450</v>
-      </c>
-      <c r="B64" s="21" t="n">
-        <f aca="false">MIN(Bewertung!$B$58,Bewertung!$B$63*(1-Bewertung!$B$59))</f>
-        <v>1150000</v>
-      </c>
-      <c r="C64" s="2"/>
+        <v>466</v>
+      </c>
+      <c r="B64" s="46" t="n">
+        <f aca="false">SUM(B52:B63)</f>
+        <v>2</v>
+      </c>
+      <c r="C64" s="47" t="n">
+        <f aca="false">SUM(C52:C63)</f>
+        <v>500000</v>
+      </c>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
       <c r="F64" s="2"/>
@@ -18867,26 +19404,21 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="16" t="s">
-        <v>451</v>
-      </c>
-      <c r="B65" s="46" t="n">
-        <f aca="false">Bewertung!$B$62/(Bewertung!$B$64+Bewertung!$B$62)</f>
-        <v>0.18942731277533</v>
-      </c>
-      <c r="C65" s="2"/>
+        <v>467</v>
+      </c>
+      <c r="B65" s="2"/>
+      <c r="C65" s="42" t="n">
+        <f aca="false">Bewertung!$B$49+Bewertung!$C$64</f>
+        <v>3000000</v>
+      </c>
       <c r="D65" s="2"/>
       <c r="E65" s="2"/>
       <c r="F65" s="2"/>
       <c r="G65" s="2"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="6" t="s">
-        <v>452</v>
-      </c>
-      <c r="B66" s="19" t="n">
-        <f aca="false">Annahmen!$B$6/(Bewertung!$B$58+Annahmen!$B$6)</f>
-        <v>0.178571428571429</v>
-      </c>
+      <c r="A66" s="2"/>
+      <c r="B66" s="2"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
@@ -18894,24 +19426,1169 @@
       <c r="G66" s="2"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="2"/>
-      <c r="B67" s="2"/>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2"/>
-      <c r="E67" s="2"/>
-      <c r="F67" s="2"/>
-      <c r="G67" s="2"/>
+      <c r="A67" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="B67" s="5"/>
+      <c r="C67" s="5"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
+      <c r="G67" s="5"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="3" t="s">
-        <v>453</v>
-      </c>
-      <c r="B68" s="2"/>
-      <c r="C68" s="2"/>
-      <c r="D68" s="2"/>
-      <c r="E68" s="2"/>
-      <c r="F68" s="2"/>
-      <c r="G68" s="2"/>
+      <c r="A68" s="12" t="s">
+        <v>469</v>
+      </c>
+      <c r="B68" s="12" t="s">
+        <v>470</v>
+      </c>
+      <c r="C68" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="D68" s="12" t="s">
+        <v>471</v>
+      </c>
+      <c r="E68" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="F68" s="12"/>
+      <c r="G68" s="12" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="6" t="s">
+        <v>473</v>
+      </c>
+      <c r="B69" s="21" t="n">
+        <f aca="false">Bewertung!$C$14</f>
+        <v>2350000</v>
+      </c>
+      <c r="C69" s="9" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D69" s="21" t="n">
+        <f aca="false">Bewertung!$E$14</f>
+        <v>900000</v>
+      </c>
+      <c r="E69" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F69" s="2"/>
+      <c r="G69" s="6" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="B70" s="21" t="n">
+        <f aca="false">Bewertung!$D$28</f>
+        <v>2950000</v>
+      </c>
+      <c r="C70" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D70" s="21" t="n">
+        <f aca="false">Bewertung!$F$28</f>
+        <v>1406250</v>
+      </c>
+      <c r="E70" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F70" s="2"/>
+      <c r="G70" s="6" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="B71" s="21" t="n">
+        <f aca="false">Bewertung!$B$39</f>
+        <v>2429877.8</v>
+      </c>
+      <c r="C71" s="9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D71" s="21" t="n">
+        <f aca="false">Bewertung!$D$39</f>
+        <v>212265.833333333</v>
+      </c>
+      <c r="E71" s="9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F71" s="2"/>
+      <c r="G71" s="6" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="6" t="s">
+        <v>479</v>
+      </c>
+      <c r="B72" s="21" t="n">
+        <f aca="false">Bewertung!$C$65</f>
+        <v>3000000</v>
+      </c>
+      <c r="C72" s="9" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D72" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" s="2"/>
+      <c r="G72" s="6" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="6" t="s">
+        <v>481</v>
+      </c>
+      <c r="B73" s="15" t="n">
+        <f aca="false">MIN(B69:B72)</f>
+        <v>2350000</v>
+      </c>
+      <c r="C73" s="2"/>
+      <c r="D73" s="15" t="n">
+        <f aca="false">MIN(D69:D71)</f>
+        <v>212265.833333333</v>
+      </c>
+      <c r="E73" s="2"/>
+      <c r="F73" s="2"/>
+      <c r="G73" s="2"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="6" t="s">
+        <v>482</v>
+      </c>
+      <c r="B74" s="15" t="n">
+        <f aca="false">MAX(B69:B72)</f>
+        <v>3000000</v>
+      </c>
+      <c r="C74" s="2"/>
+      <c r="D74" s="15" t="n">
+        <f aca="false">MAX(D69:D71)</f>
+        <v>1406250</v>
+      </c>
+      <c r="E74" s="2"/>
+      <c r="F74" s="2"/>
+      <c r="G74" s="2"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="16" t="s">
+        <v>483</v>
+      </c>
+      <c r="B75" s="24" t="n">
+        <f aca="false">SUMPRODUCT(B69:B72,C69:C72)/SUM(C69:C72)</f>
+        <v>2708475.56</v>
+      </c>
+      <c r="C75" s="2"/>
+      <c r="D75" s="17" t="n">
+        <f aca="false">SUMPRODUCT(D69:D72,E69:E72)/SUM(E69:E72)</f>
+        <v>964953.166666667</v>
+      </c>
+      <c r="E75" s="2"/>
+      <c r="F75" s="2"/>
+      <c r="G75" s="2"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="6" t="s">
+        <v>484</v>
+      </c>
+      <c r="B76" s="21" t="n">
+        <f aca="false">Bewertung!$B$75+C71*(Bewertung!$C$39-Bewertung!$B$39)/SUM(C69:C72)</f>
+        <v>2399430.5</v>
+      </c>
+      <c r="C76" s="2"/>
+      <c r="D76" s="2"/>
+      <c r="E76" s="2"/>
+      <c r="F76" s="2"/>
+      <c r="G76" s="3" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="B77" s="2"/>
+      <c r="C77" s="2"/>
+      <c r="D77" s="21" t="n">
+        <f aca="false">ROUND(Bewertung!$D$75/50000,0)*50000</f>
+        <v>950000</v>
+      </c>
+      <c r="E77" s="2"/>
+      <c r="F77" s="2"/>
+      <c r="G77" s="2"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="6" t="s">
+        <v>487</v>
+      </c>
+      <c r="B78" s="6" t="str">
+        <f aca="false">IF(AND(ROUND(SUM(C69:C72),4)=1,ROUND(SUM(E69:E72),4)=1),"OK","PRÜFEN")</f>
+        <v>OK</v>
+      </c>
+      <c r="C78" s="2"/>
+      <c r="D78" s="2"/>
+      <c r="E78" s="2"/>
+      <c r="F78" s="2"/>
+      <c r="G78" s="2"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="2"/>
+      <c r="B79" s="2"/>
+      <c r="C79" s="2"/>
+      <c r="D79" s="2"/>
+      <c r="E79" s="2"/>
+      <c r="F79" s="2"/>
+      <c r="G79" s="2"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="4" t="s">
+        <v>488</v>
+      </c>
+      <c r="B80" s="5"/>
+      <c r="C80" s="5"/>
+      <c r="D80" s="5"/>
+      <c r="E80" s="5"/>
+      <c r="F80" s="5"/>
+      <c r="G80" s="5"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="B81" s="21" t="n">
+        <f aca="false">Annahmen!$B$6</f>
+        <v>250000</v>
+      </c>
+      <c r="C81" s="2"/>
+      <c r="D81" s="2"/>
+      <c r="E81" s="2"/>
+      <c r="F81" s="2"/>
+      <c r="G81" s="2"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="16" t="s">
+        <v>489</v>
+      </c>
+      <c r="B82" s="48" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C82" s="2"/>
+      <c r="D82" s="2"/>
+      <c r="E82" s="2"/>
+      <c r="F82" s="2"/>
+      <c r="G82" s="3" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="16" t="s">
+        <v>491</v>
+      </c>
+      <c r="B83" s="23" t="n">
+        <f aca="false">Annahmen!$B$6/Bewertung!$B$82</f>
+        <v>2500000</v>
+      </c>
+      <c r="C83" s="2"/>
+      <c r="D83" s="2"/>
+      <c r="E83" s="2"/>
+      <c r="F83" s="2"/>
+      <c r="G83" s="2"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="16" t="s">
+        <v>492</v>
+      </c>
+      <c r="B84" s="42" t="n">
+        <f aca="false">Bewertung!$B$83-Annahmen!$B$6</f>
+        <v>2250000</v>
+      </c>
+      <c r="C84" s="2"/>
+      <c r="D84" s="2"/>
+      <c r="E84" s="2"/>
+      <c r="F84" s="2"/>
+      <c r="G84" s="2"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="B85" s="19" t="n">
+        <f aca="false">1-Bewertung!$B$82</f>
+        <v>0.9</v>
+      </c>
+      <c r="C85" s="2"/>
+      <c r="D85" s="2"/>
+      <c r="E85" s="2"/>
+      <c r="F85" s="2"/>
+      <c r="G85" s="2"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="B86" s="31" t="str">
+        <f aca="false">IF(ROUND(Bewertung!$B$83*Bewertung!$B$82-Annahmen!$B$6,2)=0,"OK","PRÜFEN")</f>
+        <v>OK</v>
+      </c>
+      <c r="C86" s="2"/>
+      <c r="D86" s="2"/>
+      <c r="E86" s="2"/>
+      <c r="F86" s="2"/>
+      <c r="G86" s="2"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="2"/>
+      <c r="B87" s="2"/>
+      <c r="C87" s="2"/>
+      <c r="D87" s="2"/>
+      <c r="E87" s="2"/>
+      <c r="F87" s="2"/>
+      <c r="G87" s="2"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="34" t="s">
+        <v>495</v>
+      </c>
+      <c r="B88" s="2"/>
+      <c r="C88" s="2"/>
+      <c r="D88" s="2"/>
+      <c r="E88" s="2"/>
+      <c r="F88" s="2"/>
+      <c r="G88" s="2"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="B89" s="49" t="n">
+        <f aca="false">Bewertung!$B$84/Bewertung!$B$75</f>
+        <v>0.830725605661363</v>
+      </c>
+      <c r="C89" s="2"/>
+      <c r="D89" s="2"/>
+      <c r="E89" s="2"/>
+      <c r="F89" s="2"/>
+      <c r="G89" s="2"/>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="B90" s="21" t="n">
+        <f aca="false">Bewertung!$B$84-Bewertung!$B$75</f>
+        <v>-458475.56</v>
+      </c>
+      <c r="C90" s="2"/>
+      <c r="D90" s="2"/>
+      <c r="E90" s="2"/>
+      <c r="F90" s="2"/>
+      <c r="G90" s="2"/>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="B91" s="50" t="n">
+        <f aca="false">Bewertung!$B$84/Bewertung!$B$76</f>
+        <v>0.937722513738156</v>
+      </c>
+      <c r="C91" s="2"/>
+      <c r="D91" s="2"/>
+      <c r="E91" s="2"/>
+      <c r="F91" s="2"/>
+      <c r="G91" s="2"/>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="6" t="s">
+        <v>499</v>
+      </c>
+      <c r="B92" s="50" t="n">
+        <f aca="false">Bewertung!$B$84/Bewertung!$B$73</f>
+        <v>0.957446808510638</v>
+      </c>
+      <c r="C92" s="2"/>
+      <c r="D92" s="2"/>
+      <c r="E92" s="2"/>
+      <c r="F92" s="2"/>
+      <c r="G92" s="2"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="6" t="s">
+        <v>500</v>
+      </c>
+      <c r="B93" s="50" t="n">
+        <f aca="false">Bewertung!$B$84/Bewertung!$D$75</f>
+        <v>2.3317193805088</v>
+      </c>
+      <c r="C93" s="2"/>
+      <c r="D93" s="2"/>
+      <c r="E93" s="2"/>
+      <c r="F93" s="2"/>
+      <c r="G93" s="2"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="16" t="s">
+        <v>501</v>
+      </c>
+      <c r="B94" s="31" t="str">
+        <f aca="false">IF(Bewertung!$B$84&lt;Bewertung!$B$73,"unterhalb der Gründer-Spanne – unter allen vier Methoden",IF(Bewertung!$B$84&lt;=Bewertung!$B$75,"innerhalb der Gründer-Spanne, unter dem gewichteten Mittel",IF(Bewertung!$B$84&lt;=Bewertung!$B$74,"innerhalb der Gründer-Spanne, über dem gewichteten Mittel","oberhalb der Gründer-Spanne")))</f>
+        <v>unterhalb der Gründer-Spanne – unter allen vier Methoden</v>
+      </c>
+      <c r="C94" s="2"/>
+      <c r="D94" s="2"/>
+      <c r="E94" s="2"/>
+      <c r="F94" s="2"/>
+      <c r="G94" s="2"/>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="16" t="s">
+        <v>502</v>
+      </c>
+      <c r="B95" s="31" t="str">
+        <f aca="false">IF(Bewertung!$B$84&gt;Bewertung!$D$74,"oberhalb aller konservativen Methoden",IF(Bewertung!$B$84&gt;=Bewertung!$D$75,"über dem konservativen Mittel","unter dem konservativen Mittel"))</f>
+        <v>oberhalb aller konservativen Methoden</v>
+      </c>
+      <c r="C95" s="2"/>
+      <c r="D95" s="2"/>
+      <c r="E95" s="2"/>
+      <c r="F95" s="2"/>
+      <c r="G95" s="2"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="B96" s="2"/>
+      <c r="C96" s="2"/>
+      <c r="D96" s="2"/>
+      <c r="E96" s="2"/>
+      <c r="F96" s="2"/>
+      <c r="G96" s="2"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="2"/>
+      <c r="B97" s="2"/>
+      <c r="C97" s="2"/>
+      <c r="D97" s="2"/>
+      <c r="E97" s="2"/>
+      <c r="F97" s="2"/>
+      <c r="G97" s="2"/>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="4" t="s">
+        <v>504</v>
+      </c>
+      <c r="B98" s="5"/>
+      <c r="C98" s="5"/>
+      <c r="D98" s="5"/>
+      <c r="E98" s="5"/>
+      <c r="F98" s="5"/>
+      <c r="G98" s="5"/>
+    </row>
+    <row r="99" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="12" t="s">
+        <v>505</v>
+      </c>
+      <c r="B99" s="12" t="s">
+        <v>506</v>
+      </c>
+      <c r="C99" s="12" t="s">
+        <v>507</v>
+      </c>
+      <c r="D99" s="12" t="s">
+        <v>508</v>
+      </c>
+      <c r="E99" s="12" t="s">
+        <v>509</v>
+      </c>
+      <c r="F99" s="12" t="s">
+        <v>510</v>
+      </c>
+      <c r="G99" s="12" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="9" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="B100" s="21" t="n">
+        <f aca="false">Annahmen!$B$6/A100</f>
+        <v>3125000</v>
+      </c>
+      <c r="C100" s="21" t="n">
+        <f aca="false">B100-Annahmen!$B$6</f>
+        <v>2875000</v>
+      </c>
+      <c r="D100" s="25" t="n">
+        <f aca="false">1-A100</f>
+        <v>0.92</v>
+      </c>
+      <c r="E100" s="50" t="n">
+        <f aca="false">C100/Bewertung!$B$75</f>
+        <v>1.06148271834508</v>
+      </c>
+      <c r="F100" s="50" t="n">
+        <f aca="false">C100/Bewertung!$D$75</f>
+        <v>2.9794192084279</v>
+      </c>
+      <c r="G100" s="6" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B101" s="21" t="n">
+        <f aca="false">Annahmen!$B$6/A101</f>
+        <v>2500000</v>
+      </c>
+      <c r="C101" s="39" t="n">
+        <f aca="false">B101-Annahmen!$B$6</f>
+        <v>2250000</v>
+      </c>
+      <c r="D101" s="25" t="n">
+        <f aca="false">1-A101</f>
+        <v>0.9</v>
+      </c>
+      <c r="E101" s="50" t="n">
+        <f aca="false">C101/Bewertung!$B$75</f>
+        <v>0.830725605661363</v>
+      </c>
+      <c r="F101" s="50" t="n">
+        <f aca="false">C101/Bewertung!$D$75</f>
+        <v>2.3317193805088</v>
+      </c>
+      <c r="G101" s="6" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="9" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="B102" s="21" t="n">
+        <f aca="false">Annahmen!$B$6/A102</f>
+        <v>2000000</v>
+      </c>
+      <c r="C102" s="21" t="n">
+        <f aca="false">B102-Annahmen!$B$6</f>
+        <v>1750000</v>
+      </c>
+      <c r="D102" s="25" t="n">
+        <f aca="false">1-A102</f>
+        <v>0.875</v>
+      </c>
+      <c r="E102" s="50" t="n">
+        <f aca="false">C102/Bewertung!$B$75</f>
+        <v>0.646119915514394</v>
+      </c>
+      <c r="F102" s="50" t="n">
+        <f aca="false">C102/Bewertung!$D$75</f>
+        <v>1.81355951817351</v>
+      </c>
+      <c r="G102" s="6" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="B103" s="21" t="n">
+        <f aca="false">Annahmen!$B$6/A103</f>
+        <v>1666666.66666667</v>
+      </c>
+      <c r="C103" s="21" t="n">
+        <f aca="false">B103-Annahmen!$B$6</f>
+        <v>1416666.66666667</v>
+      </c>
+      <c r="D103" s="25" t="n">
+        <f aca="false">1-A103</f>
+        <v>0.85</v>
+      </c>
+      <c r="E103" s="50" t="n">
+        <f aca="false">C103/Bewertung!$B$75</f>
+        <v>0.523049455416414</v>
+      </c>
+      <c r="F103" s="50" t="n">
+        <f aca="false">C103/Bewertung!$D$75</f>
+        <v>1.46811960994998</v>
+      </c>
+      <c r="G103" s="6" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="2"/>
+      <c r="B104" s="2"/>
+      <c r="C104" s="2"/>
+      <c r="D104" s="2"/>
+      <c r="E104" s="2"/>
+      <c r="F104" s="2"/>
+      <c r="G104" s="2"/>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="B105" s="5"/>
+      <c r="C105" s="5"/>
+      <c r="D105" s="5"/>
+      <c r="E105" s="5"/>
+      <c r="F105" s="5"/>
+      <c r="G105" s="5"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="6" t="s">
+        <v>516</v>
+      </c>
+      <c r="B106" s="21" t="n">
+        <f aca="false">Bewertung!$B$83</f>
+        <v>2500000</v>
+      </c>
+      <c r="C106" s="2"/>
+      <c r="D106" s="2"/>
+      <c r="E106" s="2"/>
+      <c r="F106" s="2"/>
+      <c r="G106" s="2"/>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="B107" s="9" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C107" s="2"/>
+      <c r="D107" s="2"/>
+      <c r="E107" s="2"/>
+      <c r="F107" s="2"/>
+      <c r="G107" s="3" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="6" t="s">
+        <v>519</v>
+      </c>
+      <c r="B108" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="C108" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="D108" s="2"/>
+      <c r="E108" s="2"/>
+      <c r="F108" s="2"/>
+      <c r="G108" s="3" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="12" t="s">
+        <v>521</v>
+      </c>
+      <c r="B109" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="C109" s="12" t="s">
+        <v>523</v>
+      </c>
+      <c r="D109" s="12" t="s">
+        <v>524</v>
+      </c>
+      <c r="E109" s="12" t="s">
+        <v>525</v>
+      </c>
+      <c r="F109" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="G109" s="12" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="B110" s="21" t="n">
+        <f aca="false">Bewertung!$B$106*A110/(1-Bewertung!$B$107)</f>
+        <v>22727272.7272727</v>
+      </c>
+      <c r="C110" s="21" t="n">
+        <f aca="false">B110/Bewertung!$B$108</f>
+        <v>5681818.18181818</v>
+      </c>
+      <c r="D110" s="21" t="n">
+        <f aca="false">B110/Bewertung!$C$108</f>
+        <v>3787878.78787879</v>
+      </c>
+      <c r="E110" s="31" t="str">
+        <f aca="false">IF('GuV 5 Jahre'!$G$15&gt;=C110,"Konservativ",IF('GuV 5 Jahre'!$G$36&gt;=C110,"Basis",IF('GuV 5 Jahre'!$G$57&gt;=C110,"Optimistisch","keines")))</f>
+        <v>Optimistisch</v>
+      </c>
+      <c r="F110" s="31" t="str">
+        <f aca="false">IF('GuV 5 Jahre'!$G$15&gt;=D110,"Konservativ",IF('GuV 5 Jahre'!$G$36&gt;=D110,"Basis",IF('GuV 5 Jahre'!$G$57&gt;=D110,"Optimistisch","keines")))</f>
+        <v>Optimistisch</v>
+      </c>
+      <c r="G110" s="3" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="B111" s="39" t="n">
+        <f aca="false">Bewertung!$B$106*A111/(1-Bewertung!$B$107)</f>
+        <v>45454545.4545455</v>
+      </c>
+      <c r="C111" s="21" t="n">
+        <f aca="false">B111/Bewertung!$B$108</f>
+        <v>11363636.3636364</v>
+      </c>
+      <c r="D111" s="21" t="n">
+        <f aca="false">B111/Bewertung!$C$108</f>
+        <v>7575757.57575758</v>
+      </c>
+      <c r="E111" s="31" t="str">
+        <f aca="false">IF('GuV 5 Jahre'!$G$15&gt;=C111,"Konservativ",IF('GuV 5 Jahre'!$G$36&gt;=C111,"Basis",IF('GuV 5 Jahre'!$G$57&gt;=C111,"Optimistisch","keines")))</f>
+        <v>keines</v>
+      </c>
+      <c r="F111" s="31" t="str">
+        <f aca="false">IF('GuV 5 Jahre'!$G$15&gt;=D111,"Konservativ",IF('GuV 5 Jahre'!$G$36&gt;=D111,"Basis",IF('GuV 5 Jahre'!$G$57&gt;=D111,"Optimistisch","keines")))</f>
+        <v>keines</v>
+      </c>
+      <c r="G111" s="3" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="2"/>
+      <c r="B112" s="2"/>
+      <c r="C112" s="2"/>
+      <c r="D112" s="2"/>
+      <c r="E112" s="2"/>
+      <c r="F112" s="2"/>
+      <c r="G112" s="2"/>
+    </row>
+    <row r="113" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="B113" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="C113" s="12" t="s">
+        <v>531</v>
+      </c>
+      <c r="D113" s="12" t="s">
+        <v>532</v>
+      </c>
+      <c r="E113" s="12" t="s">
+        <v>533</v>
+      </c>
+      <c r="F113" s="12" t="s">
+        <v>534</v>
+      </c>
+      <c r="G113" s="12" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B114" s="21" t="n">
+        <f aca="false">'GuV 5 Jahre'!$G$15</f>
+        <v>602316.6</v>
+      </c>
+      <c r="C114" s="50" t="n">
+        <f aca="false">B114*Bewertung!$B$108*(1-Bewertung!$B$107)/Bewertung!$B$106</f>
+        <v>0.530038608</v>
+      </c>
+      <c r="D114" s="50" t="n">
+        <f aca="false">B114*Bewertung!$C$108*(1-Bewertung!$B$107)/Bewertung!$B$106</f>
+        <v>0.795057912</v>
+      </c>
+      <c r="E114" s="50" t="n">
+        <f aca="false">B114*Bewertung!$C$108*(1-Bewertung!$B$36)/Bewertung!$B$106</f>
+        <v>0.867335904</v>
+      </c>
+      <c r="F114" s="19" t="n">
+        <f aca="false">B114/Bewertung!$D$111</f>
+        <v>0.0795057912</v>
+      </c>
+      <c r="G114" s="2"/>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B115" s="21" t="n">
+        <f aca="false">'GuV 5 Jahre'!$G$36</f>
+        <v>3151812.5</v>
+      </c>
+      <c r="C115" s="50" t="n">
+        <f aca="false">B115*Bewertung!$B$108*(1-Bewertung!$B$107)/Bewertung!$B$106</f>
+        <v>2.773595</v>
+      </c>
+      <c r="D115" s="50" t="n">
+        <f aca="false">B115*Bewertung!$C$108*(1-Bewertung!$B$107)/Bewertung!$B$106</f>
+        <v>4.1603925</v>
+      </c>
+      <c r="E115" s="50" t="n">
+        <f aca="false">B115*Bewertung!$C$108*(1-Bewertung!$B$36)/Bewertung!$B$106</f>
+        <v>4.53861</v>
+      </c>
+      <c r="F115" s="19" t="n">
+        <f aca="false">B115/Bewertung!$D$111</f>
+        <v>0.41603925</v>
+      </c>
+      <c r="G115" s="2"/>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B116" s="21" t="n">
+        <f aca="false">'GuV 5 Jahre'!$G$57</f>
+        <v>7444105</v>
+      </c>
+      <c r="C116" s="50" t="n">
+        <f aca="false">B116*Bewertung!$B$108*(1-Bewertung!$B$107)/Bewertung!$B$106</f>
+        <v>6.5508124</v>
+      </c>
+      <c r="D116" s="50" t="n">
+        <f aca="false">B116*Bewertung!$C$108*(1-Bewertung!$B$107)/Bewertung!$B$106</f>
+        <v>9.8262186</v>
+      </c>
+      <c r="E116" s="50" t="n">
+        <f aca="false">B116*Bewertung!$C$108*(1-Bewertung!$B$36)/Bewertung!$B$106</f>
+        <v>10.7195112</v>
+      </c>
+      <c r="F116" s="19" t="n">
+        <f aca="false">B116/Bewertung!$D$111</f>
+        <v>0.98262186</v>
+      </c>
+      <c r="G116" s="2"/>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="B117" s="2"/>
+      <c r="C117" s="2"/>
+      <c r="D117" s="2"/>
+      <c r="E117" s="2"/>
+      <c r="F117" s="2"/>
+      <c r="G117" s="2"/>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="2"/>
+      <c r="B118" s="2"/>
+      <c r="C118" s="2"/>
+      <c r="D118" s="2"/>
+      <c r="E118" s="2"/>
+      <c r="F118" s="2"/>
+      <c r="G118" s="2"/>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="B119" s="5"/>
+      <c r="C119" s="5"/>
+      <c r="D119" s="5"/>
+      <c r="E119" s="5"/>
+      <c r="F119" s="5"/>
+      <c r="G119" s="5"/>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="6" t="s">
+        <v>537</v>
+      </c>
+      <c r="B120" s="2"/>
+      <c r="C120" s="2"/>
+      <c r="D120" s="2"/>
+      <c r="E120" s="2"/>
+      <c r="F120" s="2"/>
+      <c r="G120" s="2"/>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="6" t="s">
+        <v>538</v>
+      </c>
+      <c r="B121" s="2"/>
+      <c r="C121" s="2"/>
+      <c r="D121" s="2"/>
+      <c r="E121" s="2"/>
+      <c r="F121" s="2"/>
+      <c r="G121" s="2"/>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="B122" s="2"/>
+      <c r="C122" s="2"/>
+      <c r="D122" s="2"/>
+      <c r="E122" s="2"/>
+      <c r="F122" s="2"/>
+      <c r="G122" s="2"/>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="B123" s="2"/>
+      <c r="C123" s="2"/>
+      <c r="D123" s="2"/>
+      <c r="E123" s="2"/>
+      <c r="F123" s="2"/>
+      <c r="G123" s="2"/>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="6" t="s">
+        <v>541</v>
+      </c>
+      <c r="B124" s="2"/>
+      <c r="C124" s="2"/>
+      <c r="D124" s="2"/>
+      <c r="E124" s="2"/>
+      <c r="F124" s="2"/>
+      <c r="G124" s="2"/>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="6" t="s">
+        <v>542</v>
+      </c>
+      <c r="B125" s="2"/>
+      <c r="C125" s="2"/>
+      <c r="D125" s="2"/>
+      <c r="E125" s="2"/>
+      <c r="F125" s="2"/>
+      <c r="G125" s="2"/>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="6" t="s">
+        <v>543</v>
+      </c>
+      <c r="B126" s="2"/>
+      <c r="C126" s="2"/>
+      <c r="D126" s="2"/>
+      <c r="E126" s="2"/>
+      <c r="F126" s="2"/>
+      <c r="G126" s="2"/>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="B127" s="2"/>
+      <c r="C127" s="2"/>
+      <c r="D127" s="2"/>
+      <c r="E127" s="2"/>
+      <c r="F127" s="2"/>
+      <c r="G127" s="2"/>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="2"/>
+      <c r="B128" s="2"/>
+      <c r="C128" s="2"/>
+      <c r="D128" s="2"/>
+      <c r="E128" s="2"/>
+      <c r="F128" s="2"/>
+      <c r="G128" s="2"/>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="4" t="s">
+        <v>545</v>
+      </c>
+      <c r="B129" s="5"/>
+      <c r="C129" s="5"/>
+      <c r="D129" s="5"/>
+      <c r="E129" s="5"/>
+      <c r="F129" s="5"/>
+      <c r="G129" s="5"/>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="16" t="s">
+        <v>546</v>
+      </c>
+      <c r="B130" s="7" t="n">
+        <v>2250000</v>
+      </c>
+      <c r="C130" s="31" t="str">
+        <f aca="false">IF(ROUND(Bewertung!$B$130-Bewertung!$B$84,0)=0,"= Angebot Pre-Money","weicht vom Angebot ab")</f>
+        <v>= Angebot Pre-Money</v>
+      </c>
+      <c r="D130" s="2"/>
+      <c r="E130" s="2"/>
+      <c r="F130" s="2"/>
+      <c r="G130" s="3" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="6" t="s">
+        <v>548</v>
+      </c>
+      <c r="B131" s="9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C131" s="2"/>
+      <c r="D131" s="2"/>
+      <c r="E131" s="2"/>
+      <c r="F131" s="2"/>
+      <c r="G131" s="3" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="6" t="s">
+        <v>550</v>
+      </c>
+      <c r="B132" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C132" s="2"/>
+      <c r="D132" s="2"/>
+      <c r="E132" s="2"/>
+      <c r="F132" s="2"/>
+      <c r="G132" s="2"/>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="6" t="s">
+        <v>551</v>
+      </c>
+      <c r="B133" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="C133" s="2"/>
+      <c r="D133" s="2"/>
+      <c r="E133" s="2"/>
+      <c r="F133" s="2"/>
+      <c r="G133" s="2"/>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="B134" s="21" t="n">
+        <f aca="false">Annahmen!$B$6*(1+Bewertung!$B$132*Bewertung!$B$133/12)</f>
+        <v>250000</v>
+      </c>
+      <c r="C134" s="2"/>
+      <c r="D134" s="2"/>
+      <c r="E134" s="2"/>
+      <c r="F134" s="2"/>
+      <c r="G134" s="2"/>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="6" t="s">
+        <v>553</v>
+      </c>
+      <c r="B135" s="8" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="C135" s="2"/>
+      <c r="D135" s="2"/>
+      <c r="E135" s="2"/>
+      <c r="F135" s="2"/>
+      <c r="G135" s="2"/>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="6" t="s">
+        <v>554</v>
+      </c>
+      <c r="B136" s="21" t="n">
+        <f aca="false">MIN(Bewertung!$B$130,Bewertung!$B$135*(1-Bewertung!$B$131))</f>
+        <v>2250000</v>
+      </c>
+      <c r="C136" s="2"/>
+      <c r="D136" s="2"/>
+      <c r="E136" s="2"/>
+      <c r="F136" s="2"/>
+      <c r="G136" s="2"/>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="16" t="s">
+        <v>555</v>
+      </c>
+      <c r="B137" s="51" t="n">
+        <f aca="false">Bewertung!$B$134/(Bewertung!$B$136+Bewertung!$B$134)</f>
+        <v>0.1</v>
+      </c>
+      <c r="C137" s="2"/>
+      <c r="D137" s="2"/>
+      <c r="E137" s="2"/>
+      <c r="F137" s="2"/>
+      <c r="G137" s="2"/>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="16" t="s">
+        <v>556</v>
+      </c>
+      <c r="B138" s="52" t="n">
+        <f aca="false">Annahmen!$B$6/(Bewertung!$B$130+Annahmen!$B$6)</f>
+        <v>0.1</v>
+      </c>
+      <c r="C138" s="2"/>
+      <c r="D138" s="2"/>
+      <c r="E138" s="2"/>
+      <c r="F138" s="2"/>
+      <c r="G138" s="2"/>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="6" t="s">
+        <v>557</v>
+      </c>
+      <c r="B139" s="19" t="n">
+        <f aca="false">Bewertung!$B$134/(Bewertung!$B$130+Bewertung!$B$134)</f>
+        <v>0.1</v>
+      </c>
+      <c r="C139" s="2"/>
+      <c r="D139" s="2"/>
+      <c r="E139" s="2"/>
+      <c r="F139" s="2"/>
+      <c r="G139" s="3" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="2"/>
+      <c r="B140" s="2"/>
+      <c r="C140" s="2"/>
+      <c r="D140" s="2"/>
+      <c r="E140" s="2"/>
+      <c r="F140" s="2"/>
+      <c r="G140" s="2"/>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B141" s="2"/>
+      <c r="C141" s="2"/>
+      <c r="D141" s="2"/>
+      <c r="E141" s="2"/>
+      <c r="F141" s="2"/>
+      <c r="G141" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -18940,7 +20617,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>454</v>
+        <v>560</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -18972,7 +20649,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>455</v>
+        <v>561</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -19034,52 +20711,52 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>456</v>
+        <v>562</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>457</v>
+        <v>563</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>458</v>
+        <v>564</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>459</v>
+        <v>565</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>460</v>
+        <v>566</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>461</v>
+        <v>567</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>462</v>
+        <v>568</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>463</v>
+        <v>569</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>464</v>
+        <v>570</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>465</v>
+        <v>571</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>466</v>
+        <v>572</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>467</v>
+        <v>573</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>468</v>
+        <v>574</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>469</v>
+        <v>575</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>470</v>
+        <v>576</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>471</v>
+        <v>577</v>
       </c>
       <c r="Q4" s="2"/>
       <c r="R4" s="2"/>
@@ -19098,7 +20775,7 @@
       <c r="A5" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="47" t="n">
+      <c r="B5" s="53" t="n">
         <v>0</v>
       </c>
       <c r="C5" s="40" t="n">
@@ -19111,7 +20788,7 @@
         <f aca="false">('GuV 5 Jahre'!$E$27*$D5)*('GuV 5 Jahre'!$E$28+$B5)*Annahmen!$B$13*Annahmen!$D$30*$C5*12+('GuV 5 Jahre'!$E$27*$D5)*Annahmen!$D$31*Annahmen!$B$10+'GuV 5 Jahre'!$E$33+'GuV 5 Jahre'!$E$35</f>
         <v>1038270</v>
       </c>
-      <c r="F5" s="48" t="n">
+      <c r="F5" s="54" t="n">
         <f aca="false">E5/$E$5-1</f>
         <v>0</v>
       </c>
@@ -19170,9 +20847,9 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="34" t="s">
-        <v>472</v>
-      </c>
-      <c r="B6" s="47" t="n">
+        <v>578</v>
+      </c>
+      <c r="B6" s="53" t="n">
         <v>-0.01</v>
       </c>
       <c r="C6" s="40" t="n">
@@ -19185,7 +20862,7 @@
         <f aca="false">('GuV 5 Jahre'!$E$27*$D6)*('GuV 5 Jahre'!$E$28+$B6)*Annahmen!$B$13*Annahmen!$D$30*$C6*12+('GuV 5 Jahre'!$E$27*$D6)*Annahmen!$D$31*Annahmen!$B$10+'GuV 5 Jahre'!$E$33+'GuV 5 Jahre'!$E$35</f>
         <v>847020</v>
       </c>
-      <c r="F6" s="48" t="n">
+      <c r="F6" s="54" t="n">
         <f aca="false">E6/$E$5-1</f>
         <v>-0.184200641451646</v>
       </c>
@@ -19244,9 +20921,9 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="34" t="s">
-        <v>473</v>
-      </c>
-      <c r="B7" s="47" t="n">
+        <v>579</v>
+      </c>
+      <c r="B7" s="53" t="n">
         <v>0.01</v>
       </c>
       <c r="C7" s="40" t="n">
@@ -19259,7 +20936,7 @@
         <f aca="false">('GuV 5 Jahre'!$E$27*$D7)*('GuV 5 Jahre'!$E$28+$B7)*Annahmen!$B$13*Annahmen!$D$30*$C7*12+('GuV 5 Jahre'!$E$27*$D7)*Annahmen!$D$31*Annahmen!$B$10+'GuV 5 Jahre'!$E$33+'GuV 5 Jahre'!$E$35</f>
         <v>1229520</v>
       </c>
-      <c r="F7" s="48" t="n">
+      <c r="F7" s="54" t="n">
         <f aca="false">E7/$E$5-1</f>
         <v>0.184200641451646</v>
       </c>
@@ -19318,9 +20995,9 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="34" t="s">
-        <v>474</v>
-      </c>
-      <c r="B8" s="47" t="n">
+        <v>580</v>
+      </c>
+      <c r="B8" s="53" t="n">
         <v>0</v>
       </c>
       <c r="C8" s="40" t="n">
@@ -19333,7 +21010,7 @@
         <f aca="false">('GuV 5 Jahre'!$E$27*$D8)*('GuV 5 Jahre'!$E$28+$B8)*Annahmen!$B$13*Annahmen!$D$30*$C8*12+('GuV 5 Jahre'!$E$27*$D8)*Annahmen!$D$31*Annahmen!$B$10+'GuV 5 Jahre'!$E$33+'GuV 5 Jahre'!$E$35</f>
         <v>885270</v>
       </c>
-      <c r="F8" s="48" t="n">
+      <c r="F8" s="54" t="n">
         <f aca="false">E8/$E$5-1</f>
         <v>-0.147360513161316</v>
       </c>
@@ -19392,9 +21069,9 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="34" t="s">
-        <v>475</v>
-      </c>
-      <c r="B9" s="47" t="n">
+        <v>581</v>
+      </c>
+      <c r="B9" s="53" t="n">
         <v>0</v>
       </c>
       <c r="C9" s="40" t="n">
@@ -19407,7 +21084,7 @@
         <f aca="false">('GuV 5 Jahre'!$E$27*$D9)*('GuV 5 Jahre'!$E$28+$B9)*Annahmen!$B$13*Annahmen!$D$30*$C9*12+('GuV 5 Jahre'!$E$27*$D9)*Annahmen!$D$31*Annahmen!$B$10+'GuV 5 Jahre'!$E$33+'GuV 5 Jahre'!$E$35</f>
         <v>1191270</v>
       </c>
-      <c r="F9" s="48" t="n">
+      <c r="F9" s="54" t="n">
         <f aca="false">E9/$E$5-1</f>
         <v>0.147360513161317</v>
       </c>
@@ -19466,9 +21143,9 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="34" t="s">
-        <v>476</v>
-      </c>
-      <c r="B10" s="47" t="n">
+        <v>582</v>
+      </c>
+      <c r="B10" s="53" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="40" t="n">
@@ -19481,7 +21158,7 @@
         <f aca="false">('GuV 5 Jahre'!$E$27*$D10)*('GuV 5 Jahre'!$E$28+$B10)*Annahmen!$B$13*Annahmen!$D$30*$C10*12+('GuV 5 Jahre'!$E$27*$D10)*Annahmen!$D$31*Annahmen!$B$10+'GuV 5 Jahre'!$E$33+'GuV 5 Jahre'!$E$35</f>
         <v>778845</v>
       </c>
-      <c r="F10" s="48" t="n">
+      <c r="F10" s="54" t="n">
         <f aca="false">E10/$E$5-1</f>
         <v>-0.249862752463232</v>
       </c>
@@ -19540,9 +21217,9 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="34" t="s">
-        <v>477</v>
-      </c>
-      <c r="B11" s="47" t="n">
+        <v>583</v>
+      </c>
+      <c r="B11" s="53" t="n">
         <v>0</v>
       </c>
       <c r="C11" s="40" t="n">
@@ -19555,7 +21232,7 @@
         <f aca="false">('GuV 5 Jahre'!$E$27*$D11)*('GuV 5 Jahre'!$E$28+$B11)*Annahmen!$B$13*Annahmen!$D$30*$C11*12+('GuV 5 Jahre'!$E$27*$D11)*Annahmen!$D$31*Annahmen!$B$10+'GuV 5 Jahre'!$E$33+'GuV 5 Jahre'!$E$35</f>
         <v>1297695</v>
       </c>
-      <c r="F11" s="48" t="n">
+      <c r="F11" s="54" t="n">
         <f aca="false">E11/$E$5-1</f>
         <v>0.249862752463232</v>
       </c>
@@ -19724,7 +21401,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>478</v>
+        <v>584</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -19858,7 +21535,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>479</v>
+        <v>585</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -19962,7 +21639,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>480</v>
+        <v>586</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -20066,7 +21743,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="26" t="s">
-        <v>481</v>
+        <v>587</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -20200,7 +21877,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>482</v>
+        <v>588</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -20304,7 +21981,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>483</v>
+        <v>589</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -20408,7 +22085,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="26" t="s">
-        <v>484</v>
+        <v>590</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -20542,7 +22219,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>485</v>
+        <v>591</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -20646,7 +22323,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16" t="s">
-        <v>486</v>
+        <v>592</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -20750,7 +22427,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="26" t="s">
-        <v>487</v>
+        <v>593</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -20884,7 +22561,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>488</v>
+        <v>594</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -20988,7 +22665,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16" t="s">
-        <v>489</v>
+        <v>595</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -21092,7 +22769,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="26" t="s">
-        <v>490</v>
+        <v>596</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -21226,7 +22903,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>491</v>
+        <v>597</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -21330,7 +23007,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16" t="s">
-        <v>492</v>
+        <v>598</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -21434,7 +23111,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="26" t="s">
-        <v>493</v>
+        <v>599</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -21568,7 +23245,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>494</v>
+        <v>600</v>
       </c>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -21672,7 +23349,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16" t="s">
-        <v>495</v>
+        <v>601</v>
       </c>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -21776,7 +23453,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="26" t="s">
-        <v>496</v>
+        <v>602</v>
       </c>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -21910,7 +23587,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>497</v>
+        <v>603</v>
       </c>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -22014,7 +23691,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="s">
-        <v>498</v>
+        <v>604</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -22118,7 +23795,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="26" t="s">
-        <v>499</v>
+        <v>605</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -22282,7 +23959,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>500</v>
+        <v>606</v>
       </c>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -22345,7 +24022,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>501</v>
+        <v>607</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -22371,16 +24048,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="34" t="s">
-        <v>502</v>
+        <v>608</v>
       </c>
       <c r="B3" s="34" t="s">
-        <v>503</v>
+        <v>609</v>
       </c>
       <c r="C3" s="34" t="s">
-        <v>504</v>
+        <v>610</v>
       </c>
       <c r="D3" s="34" t="s">
-        <v>505</v>
+        <v>611</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="34" t="s">
@@ -23095,7 +24772,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="46"/>
@@ -23103,7 +24780,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>506</v>
+        <v>612</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -23115,101 +24792,101 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>507</v>
+        <v>613</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>508</v>
+        <v>614</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>509</v>
+        <v>615</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>510</v>
+        <v>616</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>511</v>
+        <v>617</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>512</v>
+        <v>618</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>513</v>
+        <v>619</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>514</v>
+        <v>620</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>515</v>
+        <v>621</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>516</v>
+        <v>622</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>517</v>
+        <v>623</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>518</v>
+        <v>624</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>519</v>
+        <v>625</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>520</v>
+        <v>626</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>521</v>
+        <v>627</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>522</v>
+        <v>628</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>523</v>
+        <v>629</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>524</v>
+        <v>630</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>525</v>
+        <v>631</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>526</v>
+        <v>632</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>527</v>
+        <v>633</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>528</v>
+        <v>634</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>529</v>
+        <v>635</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>530</v>
+        <v>636</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>531</v>
+        <v>637</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>532</v>
+        <v>638</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>533</v>
+        <v>639</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23217,10 +24894,10 @@
         <v>346</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>534</v>
+        <v>640</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>535</v>
+        <v>641</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23228,10 +24905,10 @@
         <v>165</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>536</v>
+        <v>642</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>537</v>
+        <v>643</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23239,10 +24916,10 @@
         <v>348</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>538</v>
+        <v>644</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>539</v>
+        <v>645</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23250,10 +24927,10 @@
         <v>176</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>540</v>
+        <v>646</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>541</v>
+        <v>647</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23261,10 +24938,10 @@
         <v>319</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>542</v>
+        <v>648</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>543</v>
+        <v>649</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23272,10 +24949,10 @@
         <v>179</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>544</v>
+        <v>650</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>545</v>
+        <v>651</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23283,10 +24960,10 @@
         <v>181</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>546</v>
+        <v>652</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>547</v>
+        <v>653</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23294,43 +24971,43 @@
         <v>321</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>548</v>
+        <v>654</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>549</v>
+        <v>655</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>466</v>
+        <v>572</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>550</v>
+        <v>656</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>551</v>
+        <v>657</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>467</v>
+        <v>573</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>552</v>
+        <v>658</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>553</v>
+        <v>659</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>554</v>
+        <v>660</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>555</v>
+        <v>661</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>556</v>
+        <v>662</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23338,10 +25015,10 @@
         <v>270</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>557</v>
+        <v>663</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>558</v>
+        <v>664</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23349,32 +25026,32 @@
         <v>93</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>559</v>
+        <v>665</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>560</v>
+        <v>666</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>561</v>
+        <v>667</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>562</v>
+        <v>668</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>563</v>
+        <v>669</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>564</v>
+        <v>670</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>565</v>
+        <v>671</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>566</v>
+        <v>672</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23382,10 +25059,10 @@
         <v>212</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>567</v>
+        <v>673</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>568</v>
+        <v>674</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23393,7 +25070,7 @@
         <v>214</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>569</v>
+        <v>675</v>
       </c>
       <c r="C28" s="6" t="s">
         <v>214</v>
@@ -23401,79 +25078,134 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>570</v>
+        <v>676</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>571</v>
+        <v>677</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>572</v>
+        <v>678</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>573</v>
+        <v>679</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>574</v>
+        <v>680</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>575</v>
+        <v>681</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>576</v>
+        <v>505</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>577</v>
+        <v>682</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>578</v>
+        <v>683</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>579</v>
+        <v>684</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>580</v>
+        <v>685</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>581</v>
+        <v>686</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>582</v>
+        <v>687</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>583</v>
+        <v>688</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>584</v>
+        <v>689</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>342</v>
+        <v>690</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>585</v>
+        <v>691</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>586</v>
+        <v>692</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>587</v>
+        <v>693</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>588</v>
+        <v>694</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>589</v>
+        <v>695</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="s">
+        <v>696</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>697</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>699</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>700</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
+        <v>702</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>703</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>705</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6" t="s">
+        <v>707</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>708</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>709</v>
       </c>
     </row>
   </sheetData>

</xml_diff>